<commit_message>
Consolidate app and data into this single repo
Simpler for a POC: the workbook moves back to data/expenses.xlsx here and
owner/repo are detected from the Pages URL, so there is nothing to configure.
Publishing the file with the site also means the page reads without a token;
only writing needs one.

This repo is public (Pages on the free plan requires it), so the workbook is
publicly readable — documented in the README along with the two ways to
change that if this outgrows POC status.
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Expenses" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Expenses'!A1:G2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Expenses'!A1:G1</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -68,10 +68,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -437,33 +435,10 @@
         <v>Notes</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>e2edtux</v>
-      </c>
-      <c r="B2" s="1">
-        <v>45351</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Health</v>
-      </c>
-      <c r="D2" t="str">
-        <v>e2e probe — "quoted", comma, ₹ symbol</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1234.56</v>
-      </c>
-      <c r="F2" t="str">
-        <v>UPI</v>
-      </c>
-      <c r="G2" t="str">
-        <v>multi word note</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:G1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add expense: e2e probe — "quoted", comma, ₹ symbol — ₹1,234.56 (2024-02-29)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Expenses" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Expenses'!A1:G1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Expenses'!A1:G2</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -68,8 +68,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -401,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -435,10 +437,33 @@
         <v>Notes</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>e2ehp0a</v>
+      </c>
+      <c r="B2" s="1">
+        <v>45351</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Health</v>
+      </c>
+      <c r="D2" t="str">
+        <v>e2e probe — "quoted", comma, ₹ symbol</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1234.56</v>
+      </c>
+      <c r="F2" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="G2" t="str">
+        <v>multi word note</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:G2"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Delete e2e probe row
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Expenses" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Expenses'!A1:G2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Expenses'!A1:G1</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -68,10 +68,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -437,33 +435,10 @@
         <v>Notes</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>e2ehp0a</v>
-      </c>
-      <c r="B2" s="1">
-        <v>45351</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Health</v>
-      </c>
-      <c r="D2" t="str">
-        <v>e2e probe — "quoted", comma, ₹ symbol</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1234.56</v>
-      </c>
-      <c r="F2" t="str">
-        <v>UPI</v>
-      </c>
-      <c r="G2" t="str">
-        <v>multi word note</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:G1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
consistency probe: 2 rows
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -5,9 +5,6 @@
   <sheets>
     <sheet name="Expenses" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Expenses'!A1:G1</definedName>
-  </definedNames>
 </workbook>
 </file>
 
@@ -401,16 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="38.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="34.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -435,10 +423,55 @@
         <v>Notes</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>p0</v>
+      </c>
+      <c r="B2">
+        <v>45000</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Health</v>
+      </c>
+      <c r="D2" t="str">
+        <v>probe 0</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
+      </c>
+      <c r="F2" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>p1</v>
+      </c>
+      <c r="B3">
+        <v>45001</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Health</v>
+      </c>
+      <c r="D3" t="str">
+        <v>probe 1</v>
+      </c>
+      <c r="E3">
+        <v>101</v>
+      </c>
+      <c r="F3" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
consistency probe: restore empty workbook
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,55 +423,9 @@
         <v>Notes</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>p0</v>
-      </c>
-      <c r="B2">
-        <v>45000</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Health</v>
-      </c>
-      <c r="D2" t="str">
-        <v>probe 0</v>
-      </c>
-      <c r="E2">
-        <v>100</v>
-      </c>
-      <c r="F2" t="str">
-        <v>UPI</v>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>p1</v>
-      </c>
-      <c r="B3">
-        <v>45001</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Health</v>
-      </c>
-      <c r="D3" t="str">
-        <v>probe 1</v>
-      </c>
-      <c r="E3">
-        <v>101</v>
-      </c>
-      <c r="F3" t="str">
-        <v>UPI</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore the canonical empty workbook
The consistency probe left a workbook written by the probe's own minimal
builder. Replace it with the app's output, which carries the column widths,
date and currency number formats, and autofilter.
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -5,6 +5,9 @@
   <sheets>
     <sheet name="Expenses" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Expenses'!A1:G1</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -399,6 +402,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G1"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="34.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,6 +436,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G1"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Move the wedding budget into this repository
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -3,10 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Expenses" sheetId="1" r:id="rId1"/>
+    <sheet name="Budget" sheetId="1" r:id="rId1"/>
+    <sheet name="Payments" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Expenses'!A1:G1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H4</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -68,8 +71,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -401,15 +406,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:E4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="38.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -417,28 +420,308 @@
         <v>ID</v>
       </c>
       <c r="B1" t="str">
-        <v>Date</v>
+        <v>Item</v>
       </c>
       <c r="C1" t="str">
         <v>Category</v>
       </c>
       <c r="D1" t="str">
-        <v>Description</v>
+        <v>Estimated</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>168b7bbd</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Huseni Caterers</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D2" s="1">
+        <v>575000</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Reception food</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Photography &amp; Video</v>
+      </c>
+      <c r="D3" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Photography cost</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D4" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E4" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E4"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H4"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="34.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Item ID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Item</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Date</v>
       </c>
       <c r="E1" t="str">
         <v>Amount</v>
       </c>
       <c r="F1" t="str">
+        <v>Paid By</v>
+      </c>
+      <c r="G1" t="str">
         <v>Payment Method</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Notes</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>7e66fd41</v>
+      </c>
+      <c r="B2" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="D2" s="2">
+        <v>46179</v>
+      </c>
+      <c r="E2" s="1">
+        <v>15000</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Advance payment</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>e09d33db</v>
+      </c>
+      <c r="B3" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="D3" s="2">
+        <v>46220</v>
+      </c>
+      <c r="E3" s="1">
+        <v>10000</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Advance payment</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>3aeac8ad</v>
+      </c>
+      <c r="B4" t="str">
+        <v>168b7bbd</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Huseni Caterers</v>
+      </c>
+      <c r="D4" s="2">
+        <v>46233</v>
+      </c>
+      <c r="E4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Food Advance</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H4"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E5"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Item</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Estimated</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Still to pay</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Huseni Caterers</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C2" s="1">
+        <v>575000</v>
+      </c>
+      <c r="D2" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
+        <v>50000</v>
+      </c>
+      <c r="E2" s="1">
+        <f>C2-D2</f>
+        <v>525000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Photography &amp; Video</v>
+      </c>
+      <c r="C3" s="1">
+        <v>100000</v>
+      </c>
+      <c r="D3" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
+        <v>10000</v>
+      </c>
+      <c r="E3" s="1">
+        <f>C3-D3</f>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="C4" s="1">
+        <v>105000</v>
+      </c>
+      <c r="D4" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
+        <v>15000</v>
+      </c>
+      <c r="E4" s="1">
+        <f>C4-D4</f>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Total</v>
+      </c>
+      <c r="C5" s="1">
+        <f>SUM(C2:C4)</f>
+        <v>780000</v>
+      </c>
+      <c r="D5" s="1">
+        <f>SUM(D2:D4)</f>
+        <v>75000</v>
+      </c>
+      <c r="E5" s="1">
+        <f>SUM(E2:E4)</f>
+        <v>705000</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add budget item: Parag Groom 3 dress — ₹5,700.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H4</definedName>
   </definedNames>
 </workbook>
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -451,42 +451,59 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B3" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Groom 3 dress</v>
       </c>
       <c r="C3" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D3" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E3" t="str">
-        <v>Photography cost</v>
+        <v>Groom 3 dress</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Photography &amp; Video</v>
+      </c>
+      <c r="D4" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Photography cost</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
         <v>04ece648</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B5" t="str">
         <v>Soyarik mangal karyalay</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C5" t="str">
         <v>Venue &amp; Hall</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D5" s="1">
         <v>105000</v>
       </c>
-      <c r="E4" t="str">
+      <c r="E5" t="str">
         <v>venue for reception</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E4"/>
+  <autoFilter ref="A1:E5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -619,7 +636,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -666,36 +683,36 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Groom 3 dress</v>
       </c>
       <c r="B3" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C3" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>90000</v>
+        <v>5700</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B4" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C4" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
@@ -704,24 +721,43 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="C5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="D5" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
+        <v>15000</v>
+      </c>
+      <c r="E5" s="1">
+        <f>C5-D5</f>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v>Total</v>
       </c>
-      <c r="C5" s="1">
-        <f>SUM(C2:C4)</f>
-        <v>780000</v>
-      </c>
-      <c r="D5" s="1">
-        <f>SUM(D2:D4)</f>
+      <c r="C6" s="1">
+        <f>SUM(C2:C5)</f>
+        <v>785700</v>
+      </c>
+      <c r="D6" s="1">
+        <f>SUM(D2:D5)</f>
         <v>75000</v>
       </c>
-      <c r="E5" s="1">
-        <f>SUM(E2:E4)</f>
-        <v>705000</v>
+      <c r="E6" s="1">
+        <f>SUM(E2:E5)</f>
+        <v>710700</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹5,700.00 by Waheeda (mother) for Parag Groom 3 dress
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H5</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -510,7 +510,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -626,10 +626,36 @@
         <v>Food Advance</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ab012a97</v>
+      </c>
+      <c r="B5" t="str">
+        <v>113a1c1a</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Parag Groom 3 dress</v>
+      </c>
+      <c r="D5" s="2">
+        <v>46240</v>
+      </c>
+      <c r="E5" s="1">
+        <v>5700</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Waheeda (mother)</v>
+      </c>
+      <c r="G5" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H5" t="str">
+        <v>dress payment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H4"/>
+  <autoFilter ref="A1:H5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -693,11 +719,11 @@
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>5700</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>5700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -748,11 +774,11 @@
       </c>
       <c r="D6" s="1">
         <f>SUM(D2:D5)</f>
-        <v>75000</v>
+        <v>80700</v>
       </c>
       <c r="E6" s="1">
         <f>SUM(E2:E5)</f>
-        <v>710700</v>
+        <v>705000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update budget item: Parag bride 3 dress — ₹5,700.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -454,7 +454,7 @@
         <v>113a1c1a</v>
       </c>
       <c r="B3" t="str">
-        <v>Parag Groom 3 dress</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C3" t="str">
         <v>Clothing &amp; Jewellery</v>
@@ -463,7 +463,7 @@
         <v>5700</v>
       </c>
       <c r="E3" t="str">
-        <v>Groom 3 dress</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="4">
@@ -634,7 +634,7 @@
         <v>113a1c1a</v>
       </c>
       <c r="C5" t="str">
-        <v>Parag Groom 3 dress</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="D5" s="2">
         <v>46240</v>
@@ -709,7 +709,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Parag Groom 3 dress</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B3" t="str">
         <v>Clothing &amp; Jewellery</v>

</xml_diff>

<commit_message>
Add budget item: Moolchand - Bride reception dress — ₹7,604.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H5</definedName>
   </definedNames>
 </workbook>
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -451,59 +451,76 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>113a1c1a</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B3" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C3" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D3" s="1">
-        <v>5700</v>
+        <v>7604</v>
       </c>
       <c r="E3" t="str">
-        <v>bride 3 dress</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B4" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C4" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D4" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E4" t="str">
-        <v>Photography cost</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Photography &amp; Video</v>
+      </c>
+      <c r="D5" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Photography cost</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v>04ece648</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B6" t="str">
         <v>Soyarik mangal karyalay</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C6" t="str">
         <v>Venue &amp; Hall</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D6" s="1">
         <v>105000</v>
       </c>
-      <c r="E5" t="str">
+      <c r="E6" t="str">
         <v>venue for reception</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:E6"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -662,7 +679,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -709,55 +726,55 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B3" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C3" s="1">
-        <v>5700</v>
+        <v>7604</v>
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>0</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>0</v>
+        <v>7604</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B4" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C4" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B5" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C5" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
@@ -766,24 +783,43 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="C6" s="1">
+        <v>105000</v>
+      </c>
+      <c r="D6" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
+        <v>15000</v>
+      </c>
+      <c r="E6" s="1">
+        <f>C6-D6</f>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>Total</v>
       </c>
-      <c r="C6" s="1">
-        <f>SUM(C2:C5)</f>
-        <v>785700</v>
-      </c>
-      <c r="D6" s="1">
-        <f>SUM(D2:D5)</f>
+      <c r="C7" s="1">
+        <f>SUM(C2:C6)</f>
+        <v>793304</v>
+      </c>
+      <c r="D7" s="1">
+        <f>SUM(D2:D6)</f>
         <v>80700</v>
       </c>
-      <c r="E6" s="1">
-        <f>SUM(E2:E5)</f>
-        <v>705000</v>
+      <c r="E7" s="1">
+        <f>SUM(E2:E6)</f>
+        <v>712604</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹7,604.00 by Asif Sayyed (Son) for Moolchand - Bride reception dress
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H6</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -527,7 +527,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -645,34 +645,60 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ab012a97</v>
+        <v>60cefa3a</v>
       </c>
       <c r="B5" t="str">
-        <v>113a1c1a</v>
+        <v>c7e8b352</v>
       </c>
       <c r="C5" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="D5" s="2">
-        <v>46240</v>
+        <v>46233</v>
       </c>
       <c r="E5" s="1">
-        <v>5700</v>
+        <v>7604</v>
       </c>
       <c r="F5" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G5" t="str">
         <v>UPI</v>
       </c>
       <c r="H5" t="str">
+        <v>Bride reception dress</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ab012a97</v>
+      </c>
+      <c r="B6" t="str">
+        <v>113a1c1a</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Parag bride 3 dress</v>
+      </c>
+      <c r="D6" s="2">
+        <v>46240</v>
+      </c>
+      <c r="E6" s="1">
+        <v>5700</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Waheeda (mother)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H6" t="str">
         <v>dress payment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5"/>
+  <autoFilter ref="A1:H6"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -736,11 +762,11 @@
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>7604</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>7604</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -810,11 +836,11 @@
       </c>
       <c r="D7" s="1">
         <f>SUM(D2:D6)</f>
-        <v>80700</v>
+        <v>88304</v>
       </c>
       <c r="E7" s="1">
         <f>SUM(E2:E6)</f>
-        <v>712604</v>
+        <v>705000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Morya Collections - Groom wedding dress — ₹13,680.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H6</definedName>
   </definedNames>
 </workbook>
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -468,59 +468,76 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>113a1c1a</v>
+        <v>068998a3</v>
       </c>
       <c r="B4" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C4" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D4" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="E4" t="str">
-        <v>bride 3 dress</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B5" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C5" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D5" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E5" t="str">
-        <v>Photography cost</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Photography &amp; Video</v>
+      </c>
+      <c r="D6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Photography cost</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>04ece648</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B7" t="str">
         <v>Soyarik mangal karyalay</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C7" t="str">
         <v>Venue &amp; Hall</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D7" s="1">
         <v>105000</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E7" t="str">
         <v>venue for reception</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E6"/>
+  <autoFilter ref="A1:E7"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -705,7 +722,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -771,55 +788,55 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B4" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C4" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>0</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>0</v>
+        <v>13680</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B5" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C5" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B6" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C6" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
@@ -828,24 +845,43 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="C7" s="1">
+        <v>105000</v>
+      </c>
+      <c r="D7" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
+        <v>15000</v>
+      </c>
+      <c r="E7" s="1">
+        <f>C7-D7</f>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>Total</v>
       </c>
-      <c r="C7" s="1">
-        <f>SUM(C2:C6)</f>
-        <v>793304</v>
-      </c>
-      <c r="D7" s="1">
-        <f>SUM(D2:D6)</f>
+      <c r="C8" s="1">
+        <f>SUM(C2:C7)</f>
+        <v>806984</v>
+      </c>
+      <c r="D8" s="1">
+        <f>SUM(D2:D7)</f>
         <v>88304</v>
       </c>
-      <c r="E7" s="1">
-        <f>SUM(E2:E6)</f>
-        <v>705000</v>
+      <c r="E8" s="1">
+        <f>SUM(E2:E7)</f>
+        <v>718680</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹13,680.00 by Asif Sayyed (Son) for Morya Collections - Groom wedding dress
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H7</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -544,7 +544,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -688,34 +688,60 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ab012a97</v>
+        <v>2c7813c2</v>
       </c>
       <c r="B6" t="str">
-        <v>113a1c1a</v>
+        <v>068998a3</v>
       </c>
       <c r="C6" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="D6" s="2">
-        <v>46240</v>
+        <v>46233</v>
       </c>
       <c r="E6" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="F6" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G6" t="str">
         <v>UPI</v>
       </c>
       <c r="H6" t="str">
+        <v>Groom wedding dress payment</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ab012a97</v>
+      </c>
+      <c r="B7" t="str">
+        <v>113a1c1a</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Parag bride 3 dress</v>
+      </c>
+      <c r="D7" s="2">
+        <v>46240</v>
+      </c>
+      <c r="E7" s="1">
+        <v>5700</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Waheeda (mother)</v>
+      </c>
+      <c r="G7" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H7" t="str">
         <v>dress payment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H6"/>
+  <autoFilter ref="A1:H7"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -798,11 +824,11 @@
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>13680</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>13680</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -872,11 +898,11 @@
       </c>
       <c r="D8" s="1">
         <f>SUM(D2:D7)</f>
-        <v>88304</v>
+        <v>101984</v>
       </c>
       <c r="E8" s="1">
         <f>SUM(E2:E7)</f>
-        <v>718680</v>
+        <v>705000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Star Bazaar - Prewedding dress — ₹6,190.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H7</definedName>
   </definedNames>
 </workbook>
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -534,10 +534,27 @@
         <v>venue for reception</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>bd5f8d26</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D8" s="1">
+        <v>6190</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:E8"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -748,7 +765,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -890,24 +907,43 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C8" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D8" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="1">
+        <f>C8-D8</f>
+        <v>6190</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>Total</v>
       </c>
-      <c r="C8" s="1">
-        <f>SUM(C2:C7)</f>
-        <v>806984</v>
-      </c>
-      <c r="D8" s="1">
-        <f>SUM(D2:D7)</f>
+      <c r="C9" s="1">
+        <f>SUM(C2:C8)</f>
+        <v>813174</v>
+      </c>
+      <c r="D9" s="1">
+        <f>SUM(D2:D8)</f>
         <v>101984</v>
       </c>
-      <c r="E8" s="1">
-        <f>SUM(E2:E7)</f>
-        <v>705000</v>
+      <c r="E9" s="1">
+        <f>SUM(E2:E8)</f>
+        <v>711190</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹6,190.00 by Asif Sayyed (Son) for Star Bazaar - Prewedding dress
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H8</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -653,71 +653,71 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3aeac8ad</v>
+        <v>25d50b92</v>
       </c>
       <c r="B4" t="str">
-        <v>168b7bbd</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="C4" t="str">
-        <v>Huseni Caterers</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="D4" s="2">
-        <v>46233</v>
+        <v>46229</v>
       </c>
       <c r="E4" s="1">
-        <v>50000</v>
+        <v>6190</v>
       </c>
       <c r="F4" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G4" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H4" t="str">
-        <v>Food Advance</v>
+        <v>Prewedding dress payment</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>60cefa3a</v>
+        <v>3aeac8ad</v>
       </c>
       <c r="B5" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C5" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D5" s="2">
         <v>46233</v>
       </c>
       <c r="E5" s="1">
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="F5" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G5" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H5" t="str">
-        <v>Bride reception dress</v>
+        <v>Food Advance</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2c7813c2</v>
+        <v>60cefa3a</v>
       </c>
       <c r="B6" t="str">
-        <v>068998a3</v>
+        <v>c7e8b352</v>
       </c>
       <c r="C6" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="D6" s="2">
         <v>46233</v>
       </c>
       <c r="E6" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="F6" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -726,39 +726,65 @@
         <v>UPI</v>
       </c>
       <c r="H6" t="str">
-        <v>Groom wedding dress payment</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ab012a97</v>
+        <v>2c7813c2</v>
       </c>
       <c r="B7" t="str">
-        <v>113a1c1a</v>
+        <v>068998a3</v>
       </c>
       <c r="C7" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="D7" s="2">
-        <v>46240</v>
+        <v>46233</v>
       </c>
       <c r="E7" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="F7" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G7" t="str">
         <v>UPI</v>
       </c>
       <c r="H7" t="str">
+        <v>Groom wedding dress payment</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ab012a97</v>
+      </c>
+      <c r="B8" t="str">
+        <v>113a1c1a</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Parag bride 3 dress</v>
+      </c>
+      <c r="D8" s="2">
+        <v>46240</v>
+      </c>
+      <c r="E8" s="1">
+        <v>5700</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Waheeda (mother)</v>
+      </c>
+      <c r="G8" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H8" t="str">
         <v>dress payment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
+  <autoFilter ref="A1:H8"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -917,11 +943,11 @@
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>6190</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
-        <v>6190</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -934,11 +960,11 @@
       </c>
       <c r="D9" s="1">
         <f>SUM(D2:D8)</f>
-        <v>101984</v>
+        <v>108174</v>
       </c>
       <c r="E9" s="1">
         <f>SUM(E2:E8)</f>
-        <v>711190</v>
+        <v>705000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Food at shopping time — ₹2,609.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H8</definedName>
   </definedNames>
 </workbook>
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -434,127 +434,144 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>168b7bbd</v>
+        <v>070f7b33</v>
       </c>
       <c r="B2" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C2" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D2" s="1">
-        <v>575000</v>
+        <v>2609</v>
       </c>
       <c r="E2" t="str">
-        <v>Reception food</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B3" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C3" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D3" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E3" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>068998a3</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B4" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C4" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D4" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E4" t="str">
-        <v>Groom wedding dress</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>113a1c1a</v>
+        <v>068998a3</v>
       </c>
       <c r="B5" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C5" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D5" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="E5" t="str">
-        <v>bride 3 dress</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B6" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C6" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D6" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E6" t="str">
-        <v>Photography cost</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>04ece648</v>
+        <v>beb44857</v>
       </c>
       <c r="B7" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C7" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D7" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="E7" t="str">
-        <v>venue for reception</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D8" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E8" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B9" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D9" s="1">
         <v>6190</v>
       </c>
-      <c r="E8" t="str">
+      <c r="E9" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
+  <autoFilter ref="A1:E9"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -791,7 +808,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -819,55 +836,55 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B2" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C2" s="1">
-        <v>575000</v>
+        <v>2609</v>
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>525000</v>
+        <v>2609</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B3" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C3" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B4" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C4" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
@@ -876,17 +893,17 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B5" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C5" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
@@ -895,36 +912,36 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B6" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C6" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B7" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C7" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
@@ -933,43 +950,62 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B8" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C8" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C9" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D9" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E9" s="1">
+        <f>C9-D9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
         <v>Total</v>
       </c>
-      <c r="C9" s="1">
-        <f>SUM(C2:C8)</f>
-        <v>813174</v>
-      </c>
-      <c r="D9" s="1">
-        <f>SUM(D2:D8)</f>
+      <c r="C10" s="1">
+        <f>SUM(C2:C9)</f>
+        <v>815783</v>
+      </c>
+      <c r="D10" s="1">
+        <f>SUM(D2:D9)</f>
         <v>108174</v>
       </c>
-      <c r="E9" s="1">
-        <f>SUM(E2:E8)</f>
-        <v>705000</v>
+      <c r="E10" s="1">
+        <f>SUM(E2:E9)</f>
+        <v>707609</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹2,609.00 by Asif Sayyed (Son) for Food at shopping time
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H9</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -578,7 +578,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -696,71 +696,71 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>3aeac8ad</v>
+        <v>278bdc7e</v>
       </c>
       <c r="B5" t="str">
-        <v>168b7bbd</v>
+        <v>070f7b33</v>
       </c>
       <c r="C5" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="D5" s="2">
-        <v>46233</v>
+        <v>46229</v>
       </c>
       <c r="E5" s="1">
-        <v>50000</v>
+        <v>2609</v>
       </c>
       <c r="F5" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G5" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H5" t="str">
-        <v>Food Advance</v>
+        <v>Blue Nile and Seasons mall</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>60cefa3a</v>
+        <v>3aeac8ad</v>
       </c>
       <c r="B6" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C6" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D6" s="2">
         <v>46233</v>
       </c>
       <c r="E6" s="1">
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="F6" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G6" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H6" t="str">
-        <v>Bride reception dress</v>
+        <v>Food Advance</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2c7813c2</v>
+        <v>60cefa3a</v>
       </c>
       <c r="B7" t="str">
-        <v>068998a3</v>
+        <v>c7e8b352</v>
       </c>
       <c r="C7" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="D7" s="2">
         <v>46233</v>
       </c>
       <c r="E7" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="F7" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -769,39 +769,65 @@
         <v>UPI</v>
       </c>
       <c r="H7" t="str">
-        <v>Groom wedding dress payment</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ab012a97</v>
+        <v>2c7813c2</v>
       </c>
       <c r="B8" t="str">
-        <v>113a1c1a</v>
+        <v>068998a3</v>
       </c>
       <c r="C8" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="D8" s="2">
-        <v>46240</v>
+        <v>46233</v>
       </c>
       <c r="E8" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="F8" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G8" t="str">
         <v>UPI</v>
       </c>
       <c r="H8" t="str">
+        <v>Groom wedding dress payment</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ab012a97</v>
+      </c>
+      <c r="B9" t="str">
+        <v>113a1c1a</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Parag bride 3 dress</v>
+      </c>
+      <c r="D9" s="2">
+        <v>46240</v>
+      </c>
+      <c r="E9" s="1">
+        <v>5700</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Waheeda (mother)</v>
+      </c>
+      <c r="G9" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H9" t="str">
         <v>dress payment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H8"/>
+  <autoFilter ref="A1:H9"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -846,11 +872,11 @@
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>2609</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>2609</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -996,11 +1022,11 @@
       </c>
       <c r="D10" s="1">
         <f>SUM(D2:D9)</f>
-        <v>108174</v>
+        <v>110783</v>
       </c>
       <c r="E10" s="1">
         <f>SUM(E2:E9)</f>
-        <v>707609</v>
+        <v>705000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update budget item: Huseni Caterers — ₹5,75,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:E9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H9</definedName>
   </definedNames>
 </workbook>
@@ -71,9 +71,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -406,13 +407,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
     <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="34.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -429,6 +431,9 @@
         <v>Estimated</v>
       </c>
       <c r="E1" t="str">
+        <v>Contact</v>
+      </c>
+      <c r="F1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -445,7 +450,10 @@
       <c r="D2" s="1">
         <v>2609</v>
       </c>
-      <c r="E2" t="str">
+      <c r="E2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
         <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
@@ -462,7 +470,10 @@
       <c r="D3" s="1">
         <v>575000</v>
       </c>
-      <c r="E3" t="str">
+      <c r="E3" s="2" t="str">
+        <v>9226111899</v>
+      </c>
+      <c r="F3" t="str">
         <v>Reception food</v>
       </c>
     </row>
@@ -479,7 +490,10 @@
       <c r="D4" s="1">
         <v>7604</v>
       </c>
-      <c r="E4" t="str">
+      <c r="E4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
         <v>Bride reception dress</v>
       </c>
     </row>
@@ -496,7 +510,10 @@
       <c r="D5" s="1">
         <v>13680</v>
       </c>
-      <c r="E5" t="str">
+      <c r="E5" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v>Groom wedding dress</v>
       </c>
     </row>
@@ -513,7 +530,10 @@
       <c r="D6" s="1">
         <v>5700</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E6" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
         <v>bride 3 dress</v>
       </c>
     </row>
@@ -530,7 +550,10 @@
       <c r="D7" s="1">
         <v>100000</v>
       </c>
-      <c r="E7" t="str">
+      <c r="E7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
         <v>Photography cost</v>
       </c>
     </row>
@@ -547,7 +570,10 @@
       <c r="D8" s="1">
         <v>105000</v>
       </c>
-      <c r="E8" t="str">
+      <c r="E8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
         <v>venue for reception</v>
       </c>
     </row>
@@ -564,14 +590,17 @@
       <c r="D9" s="1">
         <v>6190</v>
       </c>
-      <c r="E9" t="str">
+      <c r="E9" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:F9"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -626,7 +655,7 @@
       <c r="C2" t="str">
         <v>Soyarik mangal karyalay</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>46179</v>
       </c>
       <c r="E2" s="1">
@@ -652,7 +681,7 @@
       <c r="C3" t="str">
         <v>Pratap films and Photography</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>46220</v>
       </c>
       <c r="E3" s="1">
@@ -678,7 +707,7 @@
       <c r="C4" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="3">
         <v>46229</v>
       </c>
       <c r="E4" s="1">
@@ -704,7 +733,7 @@
       <c r="C5" t="str">
         <v>Food at shopping time</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="3">
         <v>46229</v>
       </c>
       <c r="E5" s="1">
@@ -730,7 +759,7 @@
       <c r="C6" t="str">
         <v>Huseni Caterers</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="3">
         <v>46233</v>
       </c>
       <c r="E6" s="1">
@@ -756,7 +785,7 @@
       <c r="C7" t="str">
         <v>Moolchand - Bride reception dress</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="3">
         <v>46233</v>
       </c>
       <c r="E7" s="1">
@@ -782,7 +811,7 @@
       <c r="C8" t="str">
         <v>Morya Collections - Groom wedding dress</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="3">
         <v>46233</v>
       </c>
       <c r="E8" s="1">
@@ -808,7 +837,7 @@
       <c r="C9" t="str">
         <v>Parag bride 3 dress</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="3">
         <v>46240</v>
       </c>
       <c r="E9" s="1">

</xml_diff>

<commit_message>
Update payment: ₹5,700.00 by Waheeda (mother) for Parag bride 3 dress
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -699,45 +699,45 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>25d50b92</v>
+        <v>ab012a97</v>
       </c>
       <c r="B4" t="str">
-        <v>bd5f8d26</v>
+        <v>113a1c1a</v>
       </c>
       <c r="C4" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="D4" s="3">
-        <v>46229</v>
+        <v>46221</v>
       </c>
       <c r="E4" s="1">
-        <v>6190</v>
+        <v>5700</v>
       </c>
       <c r="F4" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G4" t="str">
         <v>UPI</v>
       </c>
       <c r="H4" t="str">
-        <v>Prewedding dress payment</v>
+        <v>dress payment</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>278bdc7e</v>
+        <v>25d50b92</v>
       </c>
       <c r="B5" t="str">
-        <v>070f7b33</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="C5" t="str">
-        <v>Food at shopping time</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="D5" s="3">
         <v>46229</v>
       </c>
       <c r="E5" s="1">
-        <v>2609</v>
+        <v>6190</v>
       </c>
       <c r="F5" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -746,76 +746,76 @@
         <v>UPI</v>
       </c>
       <c r="H5" t="str">
-        <v>Blue Nile and Seasons mall</v>
+        <v>Prewedding dress payment</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3aeac8ad</v>
+        <v>278bdc7e</v>
       </c>
       <c r="B6" t="str">
-        <v>168b7bbd</v>
+        <v>070f7b33</v>
       </c>
       <c r="C6" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="D6" s="3">
-        <v>46233</v>
+        <v>46229</v>
       </c>
       <c r="E6" s="1">
-        <v>50000</v>
+        <v>2609</v>
       </c>
       <c r="F6" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G6" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H6" t="str">
-        <v>Food Advance</v>
+        <v>Blue Nile and Seasons mall</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>60cefa3a</v>
+        <v>3aeac8ad</v>
       </c>
       <c r="B7" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="C7" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="D7" s="3">
         <v>46233</v>
       </c>
       <c r="E7" s="1">
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="F7" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G7" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H7" t="str">
-        <v>Bride reception dress</v>
+        <v>Food Advance</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2c7813c2</v>
+        <v>60cefa3a</v>
       </c>
       <c r="B8" t="str">
-        <v>068998a3</v>
+        <v>c7e8b352</v>
       </c>
       <c r="C8" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="D8" s="3">
         <v>46233</v>
       </c>
       <c r="E8" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="F8" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -824,33 +824,33 @@
         <v>UPI</v>
       </c>
       <c r="H8" t="str">
-        <v>Groom wedding dress payment</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ab012a97</v>
+        <v>2c7813c2</v>
       </c>
       <c r="B9" t="str">
-        <v>113a1c1a</v>
+        <v>068998a3</v>
       </c>
       <c r="C9" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="D9" s="3">
-        <v>46240</v>
+        <v>46233</v>
       </c>
       <c r="E9" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="F9" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G9" t="str">
         <v>UPI</v>
       </c>
       <c r="H9" t="str">
-        <v>dress payment</v>
+        <v>Groom wedding dress payment</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Famous Tailor - Groom Reception dress — ₹10,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H9</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -439,168 +439,188 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B2" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C2" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D2" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E2" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F2" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>168b7bbd</v>
+        <v>070f7b33</v>
       </c>
       <c r="B3" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C3" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D3" s="1">
-        <v>575000</v>
+        <v>2609</v>
       </c>
       <c r="E3" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>Reception food</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B4" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C4" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D4" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F4" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>068998a3</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B5" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C5" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D5" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E5" s="2" t="str">
         <v/>
       </c>
       <c r="F5" t="str">
-        <v>Groom wedding dress</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>113a1c1a</v>
+        <v>068998a3</v>
       </c>
       <c r="B6" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C6" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D6" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="E6" s="2" t="str">
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>bride 3 dress</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B7" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C7" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D7" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E7" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F7" t="str">
-        <v>Photography cost</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>04ece648</v>
+        <v>beb44857</v>
       </c>
       <c r="B8" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C8" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D8" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="E8" s="2" t="str">
-        <v>9850444117</v>
+        <v>9021598286</v>
       </c>
       <c r="F8" t="str">
-        <v>venue for reception</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D9" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E9" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F9" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B10" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D10" s="1">
         <v>6190</v>
       </c>
-      <c r="E9" s="2" t="str">
+      <c r="E10" s="2" t="str">
         <v/>
       </c>
-      <c r="F9" t="str">
+      <c r="F10" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F9"/>
+  <autoFilter ref="A1:F10"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -863,7 +883,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -891,74 +911,74 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B2" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C2" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>0</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>0</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B3" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C3" s="1">
-        <v>575000</v>
+        <v>2609</v>
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>2609</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B4" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C4" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B5" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C5" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
@@ -967,17 +987,17 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B6" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C6" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
@@ -986,36 +1006,36 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B7" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C7" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B8" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C8" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
@@ -1024,43 +1044,62 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B9" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C9" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C10" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D10" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E10" s="1">
+        <f>C10-D10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Total</v>
       </c>
-      <c r="C10" s="1">
-        <f>SUM(C2:C9)</f>
-        <v>815783</v>
-      </c>
-      <c r="D10" s="1">
-        <f>SUM(D2:D9)</f>
+      <c r="C11" s="1">
+        <f>SUM(C2:C10)</f>
+        <v>825783</v>
+      </c>
+      <c r="D11" s="1">
+        <f>SUM(D2:D10)</f>
         <v>110783</v>
       </c>
-      <c r="E10" s="1">
-        <f>SUM(E2:E9)</f>
-        <v>705000</v>
+      <c r="E11" s="1">
+        <f>SUM(E2:E10)</f>
+        <v>715000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹10,000.00 by Asif Sayyed (Son) for Famous Tailor - Groom Reception dress
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H10</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -627,7 +627,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -873,10 +873,36 @@
         <v>Groom wedding dress payment</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>8f87c8fa</v>
+      </c>
+      <c r="B10" t="str">
+        <v>9a8449e7</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Famous Tailor - Groom Reception dress</v>
+      </c>
+      <c r="D10" s="3">
+        <v>46240</v>
+      </c>
+      <c r="E10" s="1">
+        <v>10000</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G10" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Groom Reception dress payment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H9"/>
+  <autoFilter ref="A1:H10"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -921,11 +947,11 @@
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1090,11 +1116,11 @@
       </c>
       <c r="D11" s="1">
         <f>SUM(D2:D10)</f>
-        <v>110783</v>
+        <v>120783</v>
       </c>
       <c r="E11" s="1">
         <f>SUM(E2:E10)</f>
-        <v>715000</v>
+        <v>705000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Day night Flower Decoration - (hall) — ₹1,43,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H10</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -439,188 +439,208 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>9a8449e7</v>
+        <v>631875ca</v>
       </c>
       <c r="B2" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C2" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D2" s="1">
-        <v>10000</v>
+        <v>143000</v>
       </c>
       <c r="E2" s="2" t="str">
-        <v>9665012980</v>
+        <v>9536673041</v>
       </c>
       <c r="F2" t="str">
-        <v>Groom Reception dress</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B3" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C3" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D3" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E3" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F3" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>168b7bbd</v>
+        <v>070f7b33</v>
       </c>
       <c r="B4" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C4" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D4" s="1">
-        <v>575000</v>
+        <v>2609</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F4" t="str">
-        <v>Reception food</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B5" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C5" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D5" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E5" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F5" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>068998a3</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B6" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C6" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D6" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E6" s="2" t="str">
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>Groom wedding dress</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>113a1c1a</v>
+        <v>068998a3</v>
       </c>
       <c r="B7" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C7" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D7" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="E7" s="2" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>bride 3 dress</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B8" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C8" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D8" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E8" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>Photography cost</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>04ece648</v>
+        <v>beb44857</v>
       </c>
       <c r="B9" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C9" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D9" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="E9" s="2" t="str">
-        <v>9850444117</v>
+        <v>9021598286</v>
       </c>
       <c r="F9" t="str">
-        <v>venue for reception</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D10" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E10" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F10" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B11" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D11" s="1">
         <v>6190</v>
       </c>
-      <c r="E10" s="2" t="str">
+      <c r="E11" s="2" t="str">
         <v/>
       </c>
-      <c r="F10" t="str">
+      <c r="F11" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F10"/>
+  <autoFilter ref="A1:F11"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -909,7 +929,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -937,36 +957,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B2" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C2" s="1">
-        <v>10000</v>
+        <v>143000</v>
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>0</v>
+        <v>143000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B3" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C3" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
@@ -975,55 +995,55 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B4" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C4" s="1">
-        <v>575000</v>
+        <v>2609</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>2609</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B5" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C5" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B6" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C6" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
@@ -1032,17 +1052,17 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B7" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C7" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
@@ -1051,36 +1071,36 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B8" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C8" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B9" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C9" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
@@ -1089,43 +1109,62 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B10" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C10" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C11" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D11" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E11" s="1">
+        <f>C11-D11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>Total</v>
       </c>
-      <c r="C11" s="1">
-        <f>SUM(C2:C10)</f>
-        <v>825783</v>
-      </c>
-      <c r="D11" s="1">
-        <f>SUM(D2:D10)</f>
+      <c r="C12" s="1">
+        <f>SUM(C2:C11)</f>
+        <v>968783</v>
+      </c>
+      <c r="D12" s="1">
+        <f>SUM(D2:D11)</f>
         <v>120783</v>
       </c>
-      <c r="E11" s="1">
-        <f>SUM(E2:E10)</f>
-        <v>705000</v>
+      <c r="E12" s="1">
+        <f>SUM(E2:E11)</f>
+        <v>848000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹15,000.00 by Asif Sayyed (Son) for Day night Flower Decoration - (hall)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H11</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -647,7 +647,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -919,10 +919,36 @@
         <v>Groom Reception dress payment</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2564c285</v>
+      </c>
+      <c r="B11" t="str">
+        <v>631875ca</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Day night Flower Decoration - (hall)</v>
+      </c>
+      <c r="D11" s="3">
+        <v>46240</v>
+      </c>
+      <c r="E11" s="1">
+        <v>15000</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G11" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Advance for hall decoration</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H10"/>
+  <autoFilter ref="A1:H11"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -967,11 +993,11 @@
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>143000</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="3">
@@ -1155,11 +1181,11 @@
       </c>
       <c r="D12" s="1">
         <f>SUM(D2:D11)</f>
-        <v>120783</v>
+        <v>135783</v>
       </c>
       <c r="E12" s="1">
         <f>SUM(E2:E11)</f>
-        <v>848000</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: A S leather zone - Groom jacket — ₹3,500.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H11</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -439,208 +439,228 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>631875ca</v>
+        <v>bae4068a</v>
       </c>
       <c r="B2" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="C2" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D2" s="1">
-        <v>143000</v>
+        <v>3500</v>
       </c>
       <c r="E2" s="2" t="str">
-        <v>9536673041</v>
+        <v>08087832131</v>
       </c>
       <c r="F2" t="str">
-        <v>Hall decoration</v>
+        <v>Groom pre wedding jacket</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>9a8449e7</v>
+        <v>631875ca</v>
       </c>
       <c r="B3" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C3" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D3" s="1">
-        <v>10000</v>
+        <v>143000</v>
       </c>
       <c r="E3" s="2" t="str">
-        <v>9665012980</v>
+        <v>9536673041</v>
       </c>
       <c r="F3" t="str">
-        <v>Groom Reception dress</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B4" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C4" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D4" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F4" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>168b7bbd</v>
+        <v>070f7b33</v>
       </c>
       <c r="B5" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C5" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D5" s="1">
-        <v>575000</v>
+        <v>2609</v>
       </c>
       <c r="E5" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>Reception food</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B6" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C6" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D6" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F6" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>068998a3</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B7" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C7" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D7" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E7" s="2" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>Groom wedding dress</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>113a1c1a</v>
+        <v>068998a3</v>
       </c>
       <c r="B8" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C8" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D8" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="E8" s="2" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v>bride 3 dress</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B9" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C9" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D9" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E9" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F9" t="str">
-        <v>Photography cost</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>04ece648</v>
+        <v>beb44857</v>
       </c>
       <c r="B10" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C10" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D10" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="E10" s="2" t="str">
-        <v>9850444117</v>
+        <v>9021598286</v>
       </c>
       <c r="F10" t="str">
-        <v>venue for reception</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D11" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E11" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F11" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B12" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D12" s="1">
         <v>6190</v>
       </c>
-      <c r="E11" s="2" t="str">
+      <c r="E12" s="2" t="str">
         <v/>
       </c>
-      <c r="F11" t="str">
+      <c r="F12" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:F12"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -955,7 +975,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -983,55 +1003,55 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="B2" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C2" s="1">
-        <v>143000</v>
+        <v>3500</v>
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>128000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B3" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C3" s="1">
-        <v>10000</v>
+        <v>143000</v>
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B4" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C4" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
@@ -1040,55 +1060,55 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Huseni Caterers</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B5" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C5" s="1">
-        <v>575000</v>
+        <v>2609</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>2609</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B6" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C6" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B7" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C7" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
@@ -1097,17 +1117,17 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B8" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C8" s="1">
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>13680</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
@@ -1116,36 +1136,36 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B9" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C9" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B10" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C10" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -1154,43 +1174,62 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B11" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C11" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C12" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D12" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E12" s="1">
+        <f>C12-D12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>Total</v>
       </c>
-      <c r="C12" s="1">
-        <f>SUM(C2:C11)</f>
-        <v>968783</v>
-      </c>
-      <c r="D12" s="1">
-        <f>SUM(D2:D11)</f>
+      <c r="C13" s="1">
+        <f>SUM(C2:C12)</f>
+        <v>972283</v>
+      </c>
+      <c r="D13" s="1">
+        <f>SUM(D2:D12)</f>
         <v>135783</v>
       </c>
-      <c r="E12" s="1">
-        <f>SUM(E2:E11)</f>
-        <v>833000</v>
+      <c r="E13" s="1">
+        <f>SUM(E2:E12)</f>
+        <v>836500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹3,500.00 by Asif Sayyed (Son) for A S leather zone - Groom jacket
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H12</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -667,7 +667,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -915,19 +915,19 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>8f87c8fa</v>
+        <v>cdec8b54</v>
       </c>
       <c r="B10" t="str">
-        <v>9a8449e7</v>
+        <v>bae4068a</v>
       </c>
       <c r="C10" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="D10" s="3">
-        <v>46240</v>
+        <v>46237</v>
       </c>
       <c r="E10" s="1">
-        <v>10000</v>
+        <v>3500</v>
       </c>
       <c r="F10" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -936,24 +936,24 @@
         <v>UPI</v>
       </c>
       <c r="H10" t="str">
-        <v>Groom Reception dress payment</v>
+        <v>groom jacket</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2564c285</v>
+        <v>8f87c8fa</v>
       </c>
       <c r="B11" t="str">
-        <v>631875ca</v>
+        <v>9a8449e7</v>
       </c>
       <c r="C11" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="D11" s="3">
         <v>46240</v>
       </c>
       <c r="E11" s="1">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="F11" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -962,13 +962,39 @@
         <v>UPI</v>
       </c>
       <c r="H11" t="str">
+        <v>Groom Reception dress payment</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2564c285</v>
+      </c>
+      <c r="B12" t="str">
+        <v>631875ca</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Day night Flower Decoration - (hall)</v>
+      </c>
+      <c r="D12" s="3">
+        <v>46240</v>
+      </c>
+      <c r="E12" s="1">
+        <v>15000</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G12" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H12" t="str">
         <v>Advance for hall decoration</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:H12"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1013,11 +1039,11 @@
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1220,11 +1246,11 @@
       </c>
       <c r="D13" s="1">
         <f>SUM(D2:D12)</f>
-        <v>135783</v>
+        <v>139283</v>
       </c>
       <c r="E13" s="1">
         <f>SUM(E2:E12)</f>
-        <v>836500</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update budget item: A S leather zone - Groom jacket — ₹3,500.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -445,7 +445,7 @@
         <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="C2" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D2" s="1">
         <v>3500</v>
@@ -1032,7 +1032,7 @@
         <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="B2" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C2" s="1">
         <v>3500</v>

</xml_diff>

<commit_message>
Add budget item: Morya mojadii — ₹400.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H12</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -579,88 +579,108 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B9" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D9" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E9" s="2" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B10" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C10" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D10" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E10" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F10" t="str">
-        <v>Photography cost</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>04ece648</v>
+        <v>beb44857</v>
       </c>
       <c r="B11" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C11" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D11" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="E11" s="2" t="str">
-        <v>9850444117</v>
+        <v>9021598286</v>
       </c>
       <c r="F11" t="str">
-        <v>venue for reception</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D12" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E12" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F12" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B12" t="str">
+      <c r="B13" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D13" s="1">
         <v>6190</v>
       </c>
-      <c r="E12" s="2" t="str">
+      <c r="E13" s="2" t="str">
         <v/>
       </c>
-      <c r="F12" t="str">
+      <c r="F13" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F12"/>
+  <autoFilter ref="A1:F13"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1001,7 +1021,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1162,55 +1182,55 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C9" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>0</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>0</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B10" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C10" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B11" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C11" s="1">
-        <v>105000</v>
+        <v>100000</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -1219,43 +1239,62 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B12" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C12" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C13" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D13" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E13" s="1">
+        <f>C13-D13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
         <v>Total</v>
       </c>
-      <c r="C13" s="1">
-        <f>SUM(C2:C12)</f>
-        <v>972283</v>
-      </c>
-      <c r="D13" s="1">
-        <f>SUM(D2:D12)</f>
+      <c r="C14" s="1">
+        <f>SUM(C2:C13)</f>
+        <v>972683</v>
+      </c>
+      <c r="D14" s="1">
+        <f>SUM(D2:D13)</f>
         <v>139283</v>
       </c>
-      <c r="E13" s="1">
-        <f>SUM(E2:E12)</f>
-        <v>833000</v>
+      <c r="E14" s="1">
+        <f>SUM(E2:E13)</f>
+        <v>833400</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹400.00 by Asif Sayyed (Son) for Morya mojadii
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H13</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -687,7 +687,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1011,10 +1011,36 @@
         <v>Advance for hall decoration</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>8ec4c02a</v>
+      </c>
+      <c r="B13" t="str">
+        <v>a78dd739</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Morya mojadii</v>
+      </c>
+      <c r="D13" s="3">
+        <v>46242</v>
+      </c>
+      <c r="E13" s="1">
+        <v>400</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Shoes</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H12"/>
+  <autoFilter ref="A1:H13"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1192,11 +1218,11 @@
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1285,11 +1311,11 @@
       </c>
       <c r="D14" s="1">
         <f>SUM(D2:D13)</f>
-        <v>139283</v>
+        <v>139683</v>
       </c>
       <c r="E14" s="1">
         <f>SUM(E2:E13)</f>
-        <v>833400</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Prewedding shoot expences(lunch, fuel and other) — ₹11,840.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H13</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -639,48 +639,68 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>04ece648</v>
+        <v>6d180155</v>
       </c>
       <c r="B12" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C12" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D12" s="1">
-        <v>105000</v>
+        <v>11840</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F12" t="str">
-        <v>venue for reception</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D13" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E13" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F13" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B14" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D14" s="1">
         <v>6190</v>
       </c>
-      <c r="E13" s="2" t="str">
+      <c r="E14" s="2" t="str">
         <v/>
       </c>
-      <c r="F13" t="str">
+      <c r="F14" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F13"/>
+  <autoFilter ref="A1:F14"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1047,7 +1067,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1265,62 +1285,81 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B12" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C12" s="1">
-        <v>105000</v>
+        <v>11840</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>90000</v>
+        <v>11840</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B13" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C13" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C14" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D14" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E14" s="1">
+        <f>C14-D14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>Total</v>
       </c>
-      <c r="C14" s="1">
-        <f>SUM(C2:C13)</f>
-        <v>972683</v>
-      </c>
-      <c r="D14" s="1">
-        <f>SUM(D2:D13)</f>
+      <c r="C15" s="1">
+        <f>SUM(C2:C14)</f>
+        <v>984523</v>
+      </c>
+      <c r="D15" s="1">
+        <f>SUM(D2:D14)</f>
         <v>139683</v>
       </c>
-      <c r="E14" s="1">
-        <f>SUM(E2:E13)</f>
-        <v>833000</v>
+      <c r="E15" s="1">
+        <f>SUM(E2:E14)</f>
+        <v>844840</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹11,840.00 by Asif Sayyed (Son) for Prewedding shoot expences(lunch, fuel and other)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H14</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -707,7 +707,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1057,10 +1057,36 @@
         <v>Shoes</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>3d083a8d</v>
+      </c>
+      <c r="B14" t="str">
+        <v>6d180155</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+      </c>
+      <c r="D14" s="3">
+        <v>46244</v>
+      </c>
+      <c r="E14" s="1">
+        <v>11840</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G14" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H14" t="str">
+        <v>paid Prewedding shoot expences(lunch, fuel and other)</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H14"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1295,11 +1321,11 @@
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>11840</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>11840</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1350,11 +1376,11 @@
       </c>
       <c r="D15" s="1">
         <f>SUM(D2:D14)</f>
-        <v>139683</v>
+        <v>151523</v>
       </c>
       <c r="E15" s="1">
         <f>SUM(E2:E14)</f>
-        <v>844840</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Groom haircut and other saloon expences — ₹500.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H14</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -519,188 +519,208 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B6" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C6" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D6" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F6" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B7" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C7" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D7" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E7" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F7" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>068998a3</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B8" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C8" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D8" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E8" s="2" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v>Groom wedding dress</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B9" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D9" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E9" s="2" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B10" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D10" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E10" s="2" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B11" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C11" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D11" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E11" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F11" t="str">
-        <v>Photography cost</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B12" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C12" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D12" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F12" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>04ece648</v>
+        <v>6d180155</v>
       </c>
       <c r="B13" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C13" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D13" s="1">
-        <v>105000</v>
+        <v>11840</v>
       </c>
       <c r="E13" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F13" t="str">
-        <v>venue for reception</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D14" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E14" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F14" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B15" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D15" s="1">
         <v>6190</v>
       </c>
-      <c r="E14" s="2" t="str">
+      <c r="E15" s="2" t="str">
         <v/>
       </c>
-      <c r="F14" t="str">
+      <c r="F15" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F14"/>
+  <autoFilter ref="A1:F15"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1093,7 +1113,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1197,55 +1217,55 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B6" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C6" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>525000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B7" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C7" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B8" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C8" s="1">
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>7604</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
@@ -1254,17 +1274,17 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C9" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
@@ -1273,17 +1293,17 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C10" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -1292,100 +1312,119 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B11" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C11" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B12" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C12" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B13" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C13" s="1">
-        <v>105000</v>
+        <v>11840</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>11840</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B14" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C14" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C15" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D15" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E15" s="1">
+        <f>C15-D15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>Total</v>
       </c>
-      <c r="C15" s="1">
-        <f>SUM(C2:C14)</f>
-        <v>984523</v>
-      </c>
-      <c r="D15" s="1">
-        <f>SUM(D2:D14)</f>
+      <c r="C16" s="1">
+        <f>SUM(C2:C15)</f>
+        <v>985023</v>
+      </c>
+      <c r="D16" s="1">
+        <f>SUM(D2:D15)</f>
         <v>151523</v>
       </c>
-      <c r="E15" s="1">
-        <f>SUM(E2:E14)</f>
-        <v>833000</v>
+      <c r="E16" s="1">
+        <f>SUM(E2:E15)</f>
+        <v>833500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹500.00 by Asif Sayyed (Son) for Groom haircut and other saloon expences
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H15</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -727,7 +727,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1079,19 +1079,19 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>3d083a8d</v>
+        <v>59c568fb</v>
       </c>
       <c r="B14" t="str">
-        <v>6d180155</v>
+        <v>209d43b7</v>
       </c>
       <c r="C14" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="D14" s="3">
-        <v>46244</v>
+        <v>46243</v>
       </c>
       <c r="E14" s="1">
-        <v>11840</v>
+        <v>500</v>
       </c>
       <c r="F14" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1100,13 +1100,39 @@
         <v>UPI</v>
       </c>
       <c r="H14" t="str">
+        <v>Groom haircut and other saloon expences paid</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>3d083a8d</v>
+      </c>
+      <c r="B15" t="str">
+        <v>6d180155</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+      </c>
+      <c r="D15" s="3">
+        <v>46244</v>
+      </c>
+      <c r="E15" s="1">
+        <v>11840</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G15" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H15" t="str">
         <v>paid Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H15"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1227,11 +1253,11 @@
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1415,11 +1441,11 @@
       </c>
       <c r="D16" s="1">
         <f>SUM(D2:D15)</f>
-        <v>151523</v>
+        <v>152023</v>
       </c>
       <c r="E16" s="1">
         <f>SUM(E2:E15)</f>
-        <v>833500</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Sadi basta — ₹25,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H15</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -679,48 +679,68 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>04ece648</v>
+        <v>18d2728f</v>
       </c>
       <c r="B14" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C14" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D14" s="1">
-        <v>105000</v>
+        <v>25000</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F14" t="str">
-        <v>venue for reception</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D15" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E15" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F15" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B16" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C15" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D15" s="1">
+      <c r="C16" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D16" s="1">
         <v>6190</v>
       </c>
-      <c r="E15" s="2" t="str">
+      <c r="E16" s="2" t="str">
         <v/>
       </c>
-      <c r="F15" t="str">
+      <c r="F16" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F15"/>
+  <autoFilter ref="A1:F16"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1139,7 +1159,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1395,62 +1415,81 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B14" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C14" s="1">
-        <v>105000</v>
+        <v>25000</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>90000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B15" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C15" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C16" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D16" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E16" s="1">
+        <f>C16-D16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>Total</v>
       </c>
-      <c r="C16" s="1">
-        <f>SUM(C2:C15)</f>
-        <v>985023</v>
-      </c>
-      <c r="D16" s="1">
-        <f>SUM(D2:D15)</f>
+      <c r="C17" s="1">
+        <f>SUM(C2:C16)</f>
+        <v>1010023</v>
+      </c>
+      <c r="D17" s="1">
+        <f>SUM(D2:D16)</f>
         <v>152023</v>
       </c>
-      <c r="E16" s="1">
-        <f>SUM(E2:E15)</f>
-        <v>833000</v>
+      <c r="E17" s="1">
+        <f>SUM(E2:E16)</f>
+        <v>858000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹25,000.00 by Umar Sayyed (Father) for Sadi basta
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H16</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -747,7 +747,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1149,10 +1149,36 @@
         <v>paid Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>bd2ed5ab</v>
+      </c>
+      <c r="B16" t="str">
+        <v>18d2728f</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Sadi basta</v>
+      </c>
+      <c r="D16" s="3">
+        <v>46255</v>
+      </c>
+      <c r="E16" s="1">
+        <v>25000</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Debit Card</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Paid baste sadi</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H15"/>
+  <autoFilter ref="A1:H16"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1425,11 +1451,11 @@
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>25000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1480,11 +1506,11 @@
       </c>
       <c r="D17" s="1">
         <f>SUM(D2:D16)</f>
-        <v>152023</v>
+        <v>177023</v>
       </c>
       <c r="E17" s="1">
         <f>SUM(E2:E16)</f>
-        <v>858000</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Moolchand Sarees basta — ₹24,880.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H16</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -579,168 +579,188 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B9" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D9" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E9" s="2" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B10" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D10" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E10" s="2" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B11" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D11" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E11" s="2" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>beb44857</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B12" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C12" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D12" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F12" t="str">
-        <v>Photography cost</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B13" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C13" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D13" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E13" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F13" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B14" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C14" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D14" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E14" s="2" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>04ece648</v>
+        <v>18d2728f</v>
       </c>
       <c r="B15" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C15" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D15" s="1">
-        <v>105000</v>
+        <v>25000</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F15" t="str">
-        <v>venue for reception</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D16" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E16" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F16" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B17" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C16" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D16" s="1">
+      <c r="C17" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D17" s="1">
         <v>6190</v>
       </c>
-      <c r="E16" s="2" t="str">
+      <c r="E17" s="2" t="str">
         <v/>
       </c>
-      <c r="F16" t="str">
+      <c r="F17" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F16"/>
+  <autoFilter ref="A1:F17"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1185,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1346,36 +1366,36 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C9" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>0</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>0</v>
+        <v>24880</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C10" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -1384,17 +1404,17 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C11" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -1403,55 +1423,55 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B12" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C12" s="1">
-        <v>100000</v>
+        <v>5700</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>5700</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B13" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C13" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B14" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C14" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -1460,62 +1480,81 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B15" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C15" s="1">
-        <v>105000</v>
+        <v>25000</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>25000</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B16" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C16" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C17" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D17" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E17" s="1">
+        <f>C17-D17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
         <v>Total</v>
       </c>
-      <c r="C17" s="1">
-        <f>SUM(C2:C16)</f>
-        <v>1010023</v>
-      </c>
-      <c r="D17" s="1">
-        <f>SUM(D2:D16)</f>
+      <c r="C18" s="1">
+        <f>SUM(C2:C17)</f>
+        <v>1034903</v>
+      </c>
+      <c r="D18" s="1">
+        <f>SUM(D2:D17)</f>
         <v>177023</v>
       </c>
-      <c r="E17" s="1">
-        <f>SUM(E2:E16)</f>
-        <v>833000</v>
+      <c r="E18" s="1">
+        <f>SUM(E2:E17)</f>
+        <v>857880</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹24,880.00 by Umar Sayyed (Father) for Moolchand Sarees basta
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H17</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -767,7 +767,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1195,10 +1195,36 @@
         <v>Paid baste sadi</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>762c8b3b</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2c67b679</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Moolchand Sarees basta</v>
+      </c>
+      <c r="D17" s="3">
+        <v>46255</v>
+      </c>
+      <c r="E17" s="1">
+        <v>24880</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Debit Card</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Moolchand Sarees basta paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H17"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1376,11 +1402,11 @@
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>24880</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>24880</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1545,11 +1571,11 @@
       </c>
       <c r="D18" s="1">
         <f>SUM(D2:D17)</f>
-        <v>177023</v>
+        <v>201903</v>
       </c>
       <c r="E18" s="1">
         <f>SUM(E2:E17)</f>
-        <v>857880</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Parag Relative 20 dressed & other cloths — ₹24,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H17</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -659,108 +659,128 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B13" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C13" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D13" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E13" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F13" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B14" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C14" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D14" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F14" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B15" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C15" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D15" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E15" s="2" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>04ece648</v>
+        <v>18d2728f</v>
       </c>
       <c r="B16" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C16" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D16" s="1">
-        <v>105000</v>
+        <v>25000</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v>venue for reception</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D17" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E17" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F17" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B17" t="str">
+      <c r="B18" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C17" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D17" s="1">
+      <c r="C18" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D18" s="1">
         <v>6190</v>
       </c>
-      <c r="E17" s="2" t="str">
+      <c r="E18" s="2" t="str">
         <v/>
       </c>
-      <c r="F17" t="str">
+      <c r="F18" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F17"/>
+  <autoFilter ref="A1:F18"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F18"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1231,7 +1251,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1468,55 +1488,55 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B13" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C13" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>90000</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B14" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C14" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B15" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C15" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -1525,62 +1545,81 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B16" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C16" s="1">
-        <v>105000</v>
+        <v>25000</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>25000</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B17" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C17" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C18" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D18" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E18" s="1">
+        <f>C18-D18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v>Total</v>
       </c>
-      <c r="C18" s="1">
-        <f>SUM(C2:C17)</f>
-        <v>1034903</v>
-      </c>
-      <c r="D18" s="1">
-        <f>SUM(D2:D17)</f>
+      <c r="C19" s="1">
+        <f>SUM(C2:C18)</f>
+        <v>1058903</v>
+      </c>
+      <c r="D19" s="1">
+        <f>SUM(D2:D18)</f>
         <v>201903</v>
       </c>
-      <c r="E18" s="1">
-        <f>SUM(E2:E17)</f>
-        <v>833000</v>
+      <c r="E19" s="1">
+        <f>SUM(E2:E18)</f>
+        <v>857000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹24,000.00 by Umar Sayyed (Father) for Parag Relative 20 dressed & other cloths
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H18</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -787,7 +787,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1241,10 +1241,36 @@
         <v>Moolchand Sarees basta paid</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>04a382c3</v>
+      </c>
+      <c r="B18" t="str">
+        <v>7896f0b1</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
+      </c>
+      <c r="D18" s="3">
+        <v>46257</v>
+      </c>
+      <c r="E18" s="1">
+        <v>24000</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Debit Card</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H17"/>
+  <autoFilter ref="A1:H18"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1498,11 +1524,11 @@
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>24000</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>24000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1610,11 +1636,11 @@
       </c>
       <c r="D19" s="1">
         <f>SUM(D2:D18)</f>
-        <v>201903</v>
+        <v>225903</v>
       </c>
       <c r="E19" s="1">
         <f>SUM(E2:E18)</f>
-        <v>857000</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Famous cotton- Pathani 9 — ₹12,150.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H18</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -479,308 +479,328 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B4" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C4" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D4" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F4" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B5" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C5" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D5" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E5" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F5" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B6" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C6" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D6" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E6" s="2" t="str">
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B7" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C7" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D7" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E7" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F7" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B8" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C8" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D8" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E8" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F8" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B9" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D9" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E9" s="2" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B10" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D10" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E10" s="2" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B11" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D11" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E11" s="2" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B12" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D12" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E12" s="2" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B13" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D13" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B14" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C14" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D14" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F14" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B15" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C15" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D15" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F15" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B16" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C16" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D16" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E16" s="2" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>04ece648</v>
+        <v>18d2728f</v>
       </c>
       <c r="B17" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C17" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D17" s="1">
-        <v>105000</v>
+        <v>25000</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F17" t="str">
-        <v>venue for reception</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D18" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E18" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F18" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B18" t="str">
+      <c r="B19" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C18" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D18" s="1">
+      <c r="C19" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D19" s="1">
         <v>6190</v>
       </c>
-      <c r="E18" s="2" t="str">
+      <c r="E19" s="2" t="str">
         <v/>
       </c>
-      <c r="F18" t="str">
+      <c r="F19" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F18"/>
+  <autoFilter ref="A1:F19"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1277,7 +1297,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1343,36 +1363,36 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B4" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C4" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>0</v>
+        <v>12150</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B5" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C5" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
@@ -1381,17 +1401,17 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B6" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C6" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
@@ -1400,55 +1420,55 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B7" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C7" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B8" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C8" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C9" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
@@ -1457,17 +1477,17 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C10" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -1476,17 +1496,17 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C11" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -1495,17 +1515,17 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C12" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
@@ -1514,17 +1534,17 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C13" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -1533,55 +1553,55 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B14" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C14" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B15" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C15" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B16" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C16" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -1590,62 +1610,81 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B17" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C17" s="1">
-        <v>105000</v>
+        <v>25000</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>25000</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B18" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C18" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C19" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D19" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E19" s="1">
+        <f>C19-D19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
         <v>Total</v>
       </c>
-      <c r="C19" s="1">
-        <f>SUM(C2:C18)</f>
-        <v>1058903</v>
-      </c>
-      <c r="D19" s="1">
-        <f>SUM(D2:D18)</f>
+      <c r="C20" s="1">
+        <f>SUM(C2:C19)</f>
+        <v>1071053</v>
+      </c>
+      <c r="D20" s="1">
+        <f>SUM(D2:D19)</f>
         <v>225903</v>
       </c>
-      <c r="E19" s="1">
-        <f>SUM(E2:E18)</f>
-        <v>833000</v>
+      <c r="E20" s="1">
+        <f>SUM(E2:E19)</f>
+        <v>845150</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹12,150.00 by Umar Sayyed (Father) for Famous cotton- Pathani 9
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H19</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -807,7 +807,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1287,10 +1287,36 @@
         <v>Paid</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>b83ec348</v>
+      </c>
+      <c r="B19" t="str">
+        <v>d5fe8bfd</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Famous cotton- Pathani 9</v>
+      </c>
+      <c r="D19" s="3">
+        <v>46257</v>
+      </c>
+      <c r="E19" s="1">
+        <v>12150</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Debit Card</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Famous cotton- Pathani 9</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H18"/>
+  <autoFilter ref="A1:H19"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1373,11 +1399,11 @@
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>12150</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>12150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1675,11 +1701,11 @@
       </c>
       <c r="D20" s="1">
         <f>SUM(D2:D19)</f>
-        <v>225903</v>
+        <v>238053</v>
       </c>
       <c r="E20" s="1">
         <f>SUM(E2:E19)</f>
-        <v>845150</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Shireen Dress — ₹2,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H19</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -759,48 +759,68 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B18" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C18" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F18" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D19" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E19" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F19" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B19" t="str">
+      <c r="B20" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C19" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D19" s="1">
+      <c r="C20" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D20" s="1">
         <v>6190</v>
       </c>
-      <c r="E19" s="2" t="str">
+      <c r="E20" s="2" t="str">
         <v/>
       </c>
-      <c r="F19" t="str">
+      <c r="F20" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F19"/>
+  <autoFilter ref="A1:F20"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1323,7 +1343,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1655,62 +1675,81 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B18" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
-        <v>90000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B19" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C19" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C20" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D20" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E20" s="1">
+        <f>C20-D20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
         <v>Total</v>
       </c>
-      <c r="C20" s="1">
-        <f>SUM(C2:C19)</f>
-        <v>1071053</v>
-      </c>
-      <c r="D20" s="1">
-        <f>SUM(D2:D19)</f>
+      <c r="C21" s="1">
+        <f>SUM(C2:C20)</f>
+        <v>1073053</v>
+      </c>
+      <c r="D21" s="1">
+        <f>SUM(D2:D20)</f>
         <v>238053</v>
       </c>
-      <c r="E20" s="1">
-        <f>SUM(E2:E19)</f>
-        <v>833000</v>
+      <c r="E21" s="1">
+        <f>SUM(E2:E20)</f>
+        <v>835000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹2,000.00 by Asif Sayyed (Son) for Shireen Dress
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H20</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -827,7 +827,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1333,10 +1333,36 @@
         <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>965c1bf2</v>
+      </c>
+      <c r="B20" t="str">
+        <v>d1aee56d</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Shireen Dress</v>
+      </c>
+      <c r="D20" s="3">
+        <v>46257</v>
+      </c>
+      <c r="E20" s="1">
+        <v>2000</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G20" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Shireen Dress paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H19"/>
+  <autoFilter ref="A1:H20"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1685,11 +1711,11 @@
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1740,11 +1766,11 @@
       </c>
       <c r="D21" s="1">
         <f>SUM(D2:D20)</f>
-        <v>238053</v>
+        <v>240053</v>
       </c>
       <c r="E21" s="1">
         <f>SUM(E2:E20)</f>
-        <v>835000</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: (Mumbai Textile & Parag) Bade Abba, Anis, Navshad & Salima Dress — ₹3,750.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H20</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -439,388 +439,408 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>bae4068a</v>
+        <v>7e3ae131</v>
       </c>
       <c r="B2" t="str">
-        <v>A S leather zone - Groom jacket</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
       <c r="C2" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D2" s="1">
-        <v>3500</v>
+        <v>3750</v>
       </c>
       <c r="E2" s="2" t="str">
-        <v>08087832131</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>Groom pre wedding jacket</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>631875ca</v>
+        <v>bae4068a</v>
       </c>
       <c r="B3" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="C3" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D3" s="1">
-        <v>143000</v>
+        <v>3500</v>
       </c>
       <c r="E3" s="2" t="str">
-        <v>9536673041</v>
+        <v>08087832131</v>
       </c>
       <c r="F3" t="str">
-        <v>Hall decoration</v>
+        <v>Groom pre wedding jacket</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B4" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C4" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D4" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F4" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B5" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C5" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D5" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E5" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B6" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C6" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D6" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F6" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B7" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C7" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D7" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E7" s="2" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B8" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C8" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D8" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E8" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B9" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C9" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D9" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E9" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F9" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B10" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D10" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E10" s="2" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B11" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D11" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E11" s="2" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B12" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D12" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E12" s="2" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B13" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D13" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B14" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D14" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E14" s="2" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B15" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C15" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D15" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F15" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B16" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C16" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D16" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F16" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B17" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C17" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D17" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E17" s="2" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B18" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E18" s="2" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B19" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C19" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F19" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D20" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E20" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F20" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B20" t="str">
+      <c r="B21" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C20" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D20" s="1">
+      <c r="C21" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D21" s="1">
         <v>6190</v>
       </c>
-      <c r="E20" s="2" t="str">
+      <c r="E21" s="2" t="str">
         <v/>
       </c>
-      <c r="F20" t="str">
+      <c r="F21" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F20"/>
+  <autoFilter ref="A1:F21"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1369,7 +1389,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1397,74 +1417,74 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>A S leather zone - Groom jacket</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
       <c r="B2" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C2" s="1">
-        <v>3500</v>
+        <v>3750</v>
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>0</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="B3" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C3" s="1">
-        <v>143000</v>
+        <v>3500</v>
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>128000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B4" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C4" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B5" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C5" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
@@ -1473,17 +1493,17 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B6" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C6" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
@@ -1492,17 +1512,17 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B7" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C7" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
@@ -1511,55 +1531,55 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B8" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C8" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B9" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C9" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C10" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -1568,17 +1588,17 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C11" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -1587,17 +1607,17 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C12" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
@@ -1606,17 +1626,17 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C13" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -1625,17 +1645,17 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C14" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -1644,55 +1664,55 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B15" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C15" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B16" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C16" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B17" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C17" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -1701,17 +1721,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -1720,62 +1740,81 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B19" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B20" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C20" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C21" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D21" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E21" s="1">
+        <f>C21-D21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
         <v>Total</v>
       </c>
-      <c r="C21" s="1">
-        <f>SUM(C2:C20)</f>
-        <v>1073053</v>
-      </c>
-      <c r="D21" s="1">
-        <f>SUM(D2:D20)</f>
+      <c r="C22" s="1">
+        <f>SUM(C2:C21)</f>
+        <v>1076803</v>
+      </c>
+      <c r="D22" s="1">
+        <f>SUM(D2:D21)</f>
         <v>240053</v>
       </c>
-      <c r="E21" s="1">
-        <f>SUM(E2:E20)</f>
-        <v>833000</v>
+      <c r="E22" s="1">
+        <f>SUM(E2:E21)</f>
+        <v>836750</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹3,750.00 by Waheeda (mother) for (Mumbai Textile & Parag) Bade Abba, Anis, Navshad & Salima Dress
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H21</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -847,7 +847,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1379,10 +1379,36 @@
         <v>Shireen Dress paid</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>79903b8b</v>
+      </c>
+      <c r="B21" t="str">
+        <v>7e3ae131</v>
+      </c>
+      <c r="C21" t="str">
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
+      </c>
+      <c r="D21" s="3">
+        <v>46257</v>
+      </c>
+      <c r="E21" s="1">
+        <v>3750</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Waheeda (mother)</v>
+      </c>
+      <c r="G21" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H21" t="str">
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H21"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1427,11 +1453,11 @@
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>3750</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>3750</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1805,11 +1831,11 @@
       </c>
       <c r="D22" s="1">
         <f>SUM(D2:D21)</f>
-        <v>240053</v>
+        <v>243803</v>
       </c>
       <c r="E22" s="1">
         <f>SUM(E2:E21)</f>
-        <v>836750</v>
+        <v>833000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: (Famous & Libas Tailor)Silaee for Abba, Didi, Asif & irfan Bhaijan — ₹11,300.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H21</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -439,408 +439,428 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>7e3ae131</v>
+        <v>4e1fe7bf</v>
       </c>
       <c r="B2" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
+        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
       </c>
       <c r="C2" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D2" s="1">
-        <v>3750</v>
+        <v>11300</v>
       </c>
       <c r="E2" s="2" t="str">
-        <v/>
+        <v>9665012980/ 9172324233</v>
       </c>
       <c r="F2" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
+        <v>Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>bae4068a</v>
+        <v>7e3ae131</v>
       </c>
       <c r="B3" t="str">
-        <v>A S leather zone - Groom jacket</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
       <c r="C3" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D3" s="1">
-        <v>3500</v>
+        <v>3750</v>
       </c>
       <c r="E3" s="2" t="str">
-        <v>08087832131</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>Groom pre wedding jacket</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>631875ca</v>
+        <v>bae4068a</v>
       </c>
       <c r="B4" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="C4" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D4" s="1">
-        <v>143000</v>
+        <v>3500</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v>9536673041</v>
+        <v>08087832131</v>
       </c>
       <c r="F4" t="str">
-        <v>Hall decoration</v>
+        <v>Groom pre wedding jacket</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B5" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C5" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D5" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E5" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F5" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B6" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C6" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D6" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F6" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B7" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C7" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D7" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E7" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F7" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B8" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C8" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D8" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E8" s="2" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B9" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C9" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D9" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E9" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F9" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B10" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C10" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D10" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E10" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F10" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B11" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D11" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E11" s="2" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B12" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D12" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E12" s="2" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B13" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D13" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B14" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D14" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E14" s="2" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B15" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D15" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E15" s="2" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B16" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C16" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D16" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B17" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C17" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D17" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F17" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B18" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C18" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D18" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E18" s="2" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B19" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E19" s="2" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B20" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C20" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F20" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D21" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E21" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F21" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B21" t="str">
+      <c r="B22" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C21" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D21" s="1">
+      <c r="C22" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D22" s="1">
         <v>6190</v>
       </c>
-      <c r="E21" s="2" t="str">
+      <c r="E22" s="2" t="str">
         <v/>
       </c>
-      <c r="F21" t="str">
+      <c r="F22" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F21"/>
+  <autoFilter ref="A1:F22"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F22"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1415,7 +1435,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1443,36 +1463,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
+        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
       </c>
       <c r="B2" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C2" s="1">
-        <v>3750</v>
+        <v>11300</v>
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>3750</v>
+        <v>0</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>0</v>
+        <v>11300</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>A S leather zone - Groom jacket</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
       <c r="B3" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C3" s="1">
-        <v>3500</v>
+        <v>3750</v>
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>3500</v>
+        <v>3750</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
@@ -1481,55 +1501,55 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="B4" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C4" s="1">
-        <v>143000</v>
+        <v>3500</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>128000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B5" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C5" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B6" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C6" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
@@ -1538,17 +1558,17 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B7" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C7" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
@@ -1557,17 +1577,17 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B8" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C8" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
@@ -1576,55 +1596,55 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B9" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C9" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B10" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C10" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C11" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -1633,17 +1653,17 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C12" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
@@ -1652,17 +1672,17 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C13" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -1671,17 +1691,17 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C14" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -1690,17 +1710,17 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C15" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -1709,55 +1729,55 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B16" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C16" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B17" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C17" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B18" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C18" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -1766,17 +1786,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -1785,62 +1805,81 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B20" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B21" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C21" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C22" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D22" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E22" s="1">
+        <f>C22-D22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
         <v>Total</v>
       </c>
-      <c r="C22" s="1">
-        <f>SUM(C2:C21)</f>
-        <v>1076803</v>
-      </c>
-      <c r="D22" s="1">
-        <f>SUM(D2:D21)</f>
+      <c r="C23" s="1">
+        <f>SUM(C2:C22)</f>
+        <v>1088103</v>
+      </c>
+      <c r="D23" s="1">
+        <f>SUM(D2:D22)</f>
         <v>243803</v>
       </c>
-      <c r="E22" s="1">
-        <f>SUM(E2:E21)</f>
-        <v>833000</v>
+      <c r="E23" s="1">
+        <f>SUM(E2:E22)</f>
+        <v>844300</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹1,000.00 by Umar Sayyed (Father) for (Famous & Libas Tailor)Silaee for Abba, Didi, Asif & irfan Bhaijan
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H22</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -867,7 +867,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1425,10 +1425,36 @@
         <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>109c6f27</v>
+      </c>
+      <c r="B22" t="str">
+        <v>4e1fe7bf</v>
+      </c>
+      <c r="C22" t="str">
+        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
+      </c>
+      <c r="D22" s="3">
+        <v>46257</v>
+      </c>
+      <c r="E22" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H22" t="str">
+        <v>advance</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H21"/>
+  <autoFilter ref="A1:H22"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1473,11 +1499,11 @@
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>11300</v>
+        <v>10300</v>
       </c>
     </row>
     <row r="3">
@@ -1870,11 +1896,11 @@
       </c>
       <c r="D23" s="1">
         <f>SUM(D2:D22)</f>
-        <v>243803</v>
+        <v>244803</v>
       </c>
       <c r="E23" s="1">
         <f>SUM(E2:E22)</f>
-        <v>844300</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update budget item: (Mumbai Textile & Parag) Bade Abba, Anis, Navshad & Salima Dress — ₹4,080.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -468,7 +468,7 @@
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D3" s="1">
-        <v>3750</v>
+        <v>4080</v>
       </c>
       <c r="E3" s="2" t="str">
         <v/>
@@ -1514,7 +1514,7 @@
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C3" s="1">
-        <v>3750</v>
+        <v>4080</v>
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>0</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="C23" s="1">
         <f>SUM(C2:C22)</f>
-        <v>1088103</v>
+        <v>1088433</v>
       </c>
       <c r="D23" s="1">
         <f>SUM(D2:D22)</f>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="E23" s="1">
         <f>SUM(E2:E22)</f>
-        <v>843300</v>
+        <v>843630</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update payment: ₹4,080.00 by Waheeda (mother) for (Mumbai Textile & Parag) Bade Abba, Anis, Navshad & Salima Dress
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -1413,7 +1413,7 @@
         <v>46257</v>
       </c>
       <c r="E21" s="1">
-        <v>3750</v>
+        <v>4080</v>
       </c>
       <c r="F21" t="str">
         <v>Waheeda (mother)</v>
@@ -1518,11 +1518,11 @@
       </c>
       <c r="D3" s="1">
         <f>SUMIF('Payments'!$C:$C,$A3,'Payments'!$E:$E)</f>
-        <v>3750</v>
+        <v>4080</v>
       </c>
       <c r="E3" s="1">
         <f>C3-D3</f>
-        <v>330</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1896,11 +1896,11 @@
       </c>
       <c r="D23" s="1">
         <f>SUM(D2:D22)</f>
-        <v>244803</v>
+        <v>245133</v>
       </c>
       <c r="E23" s="1">
         <f>SUM(E2:E22)</f>
-        <v>843630</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: 23 Aug Basta lunch at Shahidawat — ₹2,545.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H22</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -479,388 +479,408 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>bae4068a</v>
+        <v>1bb495b6</v>
       </c>
       <c r="B4" t="str">
-        <v>A S leather zone - Groom jacket</v>
+        <v>23 Aug Basta lunch at Shahidawat</v>
       </c>
       <c r="C4" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D4" s="1">
-        <v>3500</v>
+        <v>2545</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v>08087832131</v>
+        <v/>
       </c>
       <c r="F4" t="str">
-        <v>Groom pre wedding jacket</v>
+        <v>23 Aug Basta lunch</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>631875ca</v>
+        <v>bae4068a</v>
       </c>
       <c r="B5" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="C5" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D5" s="1">
-        <v>143000</v>
+        <v>3500</v>
       </c>
       <c r="E5" s="2" t="str">
-        <v>9536673041</v>
+        <v>08087832131</v>
       </c>
       <c r="F5" t="str">
-        <v>Hall decoration</v>
+        <v>Groom pre wedding jacket</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B6" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C6" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D6" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F6" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B7" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C7" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D7" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E7" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F7" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B8" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C8" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D8" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E8" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F8" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B9" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C9" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D9" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E9" s="2" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B10" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C10" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D10" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E10" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F10" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B11" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C11" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D11" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E11" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F11" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B12" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D12" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E12" s="2" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B13" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D13" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B14" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D14" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E14" s="2" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B15" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D15" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E15" s="2" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B16" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D16" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E16" s="2" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B17" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C17" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D17" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F17" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B18" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C18" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D18" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F18" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B19" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C19" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D19" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E19" s="2" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B20" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E20" s="2" t="str">
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B21" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C21" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D21" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F21" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D22" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E22" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F22" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B22" t="str">
+      <c r="B23" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C22" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D22" s="1">
+      <c r="C23" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D23" s="1">
         <v>6190</v>
       </c>
-      <c r="E22" s="2" t="str">
+      <c r="E23" s="2" t="str">
         <v/>
       </c>
-      <c r="F22" t="str">
+      <c r="F23" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F22"/>
+  <autoFilter ref="A1:F23"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1461,7 +1481,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1527,74 +1547,74 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>A S leather zone - Groom jacket</v>
+        <v>23 Aug Basta lunch at Shahidawat</v>
       </c>
       <c r="B4" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C4" s="1">
-        <v>3500</v>
+        <v>2545</v>
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>0</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>A S leather zone - Groom jacket</v>
       </c>
       <c r="B5" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C5" s="1">
-        <v>143000</v>
+        <v>3500</v>
       </c>
       <c r="D5" s="1">
         <f>SUMIF('Payments'!$C:$C,$A5,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>3500</v>
       </c>
       <c r="E5" s="1">
         <f>C5-D5</f>
-        <v>128000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B6" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C6" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B7" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C7" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
@@ -1603,17 +1623,17 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B8" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C8" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
@@ -1622,17 +1642,17 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B9" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C9" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
@@ -1641,55 +1661,55 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B10" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C10" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B11" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C11" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C12" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
@@ -1698,17 +1718,17 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C13" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -1717,17 +1737,17 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C14" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -1736,17 +1756,17 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C15" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -1755,17 +1775,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C16" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -1774,55 +1794,55 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B17" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C17" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B18" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C18" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B19" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C19" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -1831,17 +1851,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -1850,62 +1870,81 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B21" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C21" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B22" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C22" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C23" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D23" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E23" s="1">
+        <f>C23-D23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>Total</v>
       </c>
-      <c r="C23" s="1">
-        <f>SUM(C2:C22)</f>
-        <v>1088433</v>
-      </c>
-      <c r="D23" s="1">
-        <f>SUM(D2:D22)</f>
+      <c r="C24" s="1">
+        <f>SUM(C2:C23)</f>
+        <v>1090978</v>
+      </c>
+      <c r="D24" s="1">
+        <f>SUM(D2:D23)</f>
         <v>245133</v>
       </c>
-      <c r="E23" s="1">
-        <f>SUM(E2:E22)</f>
-        <v>843300</v>
+      <c r="E24" s="1">
+        <f>SUM(E2:E23)</f>
+        <v>845845</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹2,545.00 by Asif Sayyed (Son) for 23 Aug Basta lunch at Shahidawat
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H23</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -887,7 +887,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1471,10 +1471,36 @@
         <v>advance</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>b5b081de</v>
+      </c>
+      <c r="B23" t="str">
+        <v>1bb495b6</v>
+      </c>
+      <c r="C23" t="str">
+        <v>23 Aug Basta lunch at Shahidawat</v>
+      </c>
+      <c r="D23" s="3">
+        <v>46257</v>
+      </c>
+      <c r="E23" s="1">
+        <v>2545</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G23" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H23" t="str">
+        <v>23 Aug Basta lunch paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H22"/>
+  <autoFilter ref="A1:H23"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1557,11 +1583,11 @@
       </c>
       <c r="D4" s="1">
         <f>SUMIF('Payments'!$C:$C,$A4,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>2545</v>
       </c>
       <c r="E4" s="1">
         <f>C4-D4</f>
-        <v>2545</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1935,11 +1961,11 @@
       </c>
       <c r="D24" s="1">
         <f>SUM(D2:D23)</f>
-        <v>245133</v>
+        <v>247678</v>
       </c>
       <c r="E24" s="1">
         <f>SUM(E2:E23)</f>
-        <v>845845</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Arbiya Bangals — ₹550.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H23</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -519,368 +519,388 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>631875ca</v>
+        <v>a036f9f7</v>
       </c>
       <c r="B6" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="C6" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D6" s="1">
-        <v>143000</v>
+        <v>550</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F6" t="str">
-        <v>Hall decoration</v>
+        <v>Arbiya Bangals</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B7" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C7" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D7" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E7" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F7" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B8" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C8" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D8" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E8" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B9" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C9" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D9" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E9" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F9" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B10" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C10" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D10" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E10" s="2" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B11" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C11" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D11" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E11" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F11" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B12" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C12" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D12" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F12" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B13" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D13" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B14" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D14" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E14" s="2" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B15" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D15" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E15" s="2" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B16" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D16" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E16" s="2" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B17" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D17" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E17" s="2" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B18" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C18" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F18" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B19" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C19" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D19" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F19" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B20" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C20" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D20" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E20" s="2" t="str">
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B21" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D21" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E21" s="2" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B22" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C22" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D22" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F22" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D23" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E23" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F23" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B23" t="str">
+      <c r="B24" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C23" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D23" s="1">
+      <c r="C24" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D24" s="1">
         <v>6190</v>
       </c>
-      <c r="E23" s="2" t="str">
+      <c r="E24" s="2" t="str">
         <v/>
       </c>
-      <c r="F23" t="str">
+      <c r="F24" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F23"/>
+  <autoFilter ref="A1:F24"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1507,7 +1527,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1611,55 +1631,55 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="B6" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C6" s="1">
-        <v>143000</v>
+        <v>550</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>128000</v>
+        <v>550</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B7" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C7" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B8" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C8" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
@@ -1668,17 +1688,17 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B9" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C9" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
@@ -1687,17 +1707,17 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B10" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C10" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -1706,55 +1726,55 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B11" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C11" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B12" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C12" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C13" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -1763,17 +1783,17 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C14" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -1782,17 +1802,17 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C15" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -1801,17 +1821,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C16" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -1820,17 +1840,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C17" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -1839,55 +1859,55 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B18" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B19" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C19" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B20" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C20" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -1896,17 +1916,17 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C21" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -1915,62 +1935,81 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B22" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C22" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B23" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C23" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C24" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D24" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E24" s="1">
+        <f>C24-D24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
         <v>Total</v>
       </c>
-      <c r="C24" s="1">
-        <f>SUM(C2:C23)</f>
-        <v>1090978</v>
-      </c>
-      <c r="D24" s="1">
-        <f>SUM(D2:D23)</f>
+      <c r="C25" s="1">
+        <f>SUM(C2:C24)</f>
+        <v>1091528</v>
+      </c>
+      <c r="D25" s="1">
+        <f>SUM(D2:D24)</f>
         <v>247678</v>
       </c>
-      <c r="E24" s="1">
-        <f>SUM(E2:E23)</f>
-        <v>843300</v>
+      <c r="E25" s="1">
+        <f>SUM(E2:E24)</f>
+        <v>843850</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹550.00 by Asif Sayyed (Son) for Arbiya Bangals
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H24</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -907,7 +907,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1517,10 +1517,36 @@
         <v>23 Aug Basta lunch paid</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>de8adadf</v>
+      </c>
+      <c r="B24" t="str">
+        <v>a036f9f7</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Arbiya Bangals</v>
+      </c>
+      <c r="D24" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E24" s="1">
+        <v>550</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G24" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Bangal</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H23"/>
+  <autoFilter ref="A1:H24"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1641,11 +1667,11 @@
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>550</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>550</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2000,11 +2026,11 @@
       </c>
       <c r="D25" s="1">
         <f>SUM(D2:D24)</f>
-        <v>247678</v>
+        <v>248228</v>
       </c>
       <c r="E25" s="1">
         <f>SUM(E2:E24)</f>
-        <v>843850</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Arbiya & Didi Sangle — ₹1,300.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H24</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -519,388 +519,408 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>a036f9f7</v>
+        <v>985ce939</v>
       </c>
       <c r="B6" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
       <c r="C6" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D6" s="1">
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="E6" s="2" t="str">
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>631875ca</v>
+        <v>a036f9f7</v>
       </c>
       <c r="B7" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="C7" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D7" s="1">
-        <v>143000</v>
+        <v>550</v>
       </c>
       <c r="E7" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F7" t="str">
-        <v>Hall decoration</v>
+        <v>Arbiya Bangals</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B8" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C8" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D8" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E8" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F8" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B9" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D9" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E9" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F9" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B10" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C10" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D10" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E10" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F10" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B11" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C11" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D11" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E11" s="2" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B12" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C12" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D12" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F12" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>c7e8b352</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B13" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C13" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D13" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="E13" s="2" t="str">
-        <v/>
+        <v>9226111899</v>
       </c>
       <c r="F13" t="str">
-        <v>Bride reception dress</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B14" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D14" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E14" s="2" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B15" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D15" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E15" s="2" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B16" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D16" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E16" s="2" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B17" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D17" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E17" s="2" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B18" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E18" s="2" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B19" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C19" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F19" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B20" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C20" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D20" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F20" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B21" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C21" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D21" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E21" s="2" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B22" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D22" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E22" s="2" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B23" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C23" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D23" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F23" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D24" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E24" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F24" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B24" t="str">
+      <c r="B25" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C24" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D24" s="1">
+      <c r="C25" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D25" s="1">
         <v>6190</v>
       </c>
-      <c r="E24" s="2" t="str">
+      <c r="E25" s="2" t="str">
         <v/>
       </c>
-      <c r="F24" t="str">
+      <c r="F25" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F24"/>
+  <autoFilter ref="A1:F25"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F25"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1553,7 +1573,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1657,74 +1677,74 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
       <c r="B6" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C6" s="1">
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>0</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="B7" t="str">
-        <v>Decoration</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C7" s="1">
-        <v>143000</v>
+        <v>550</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>550</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
-        <v>128000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B8" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C8" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B9" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C9" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
@@ -1733,17 +1753,17 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B10" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C10" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -1752,17 +1772,17 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B11" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C11" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -1771,55 +1791,55 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B12" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C12" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B13" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C13" s="1">
-        <v>7604</v>
+        <v>575000</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>50000</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C14" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -1828,17 +1848,17 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C15" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -1847,17 +1867,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C16" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -1866,17 +1886,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C17" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -1885,17 +1905,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -1904,55 +1924,55 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B19" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B20" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C20" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B21" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C21" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -1961,17 +1981,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C22" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -1980,62 +2000,81 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B23" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C23" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B24" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C24" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C25" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D25" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E25" s="1">
+        <f>C25-D25</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
         <v>Total</v>
       </c>
-      <c r="C25" s="1">
-        <f>SUM(C2:C24)</f>
-        <v>1091528</v>
-      </c>
-      <c r="D25" s="1">
-        <f>SUM(D2:D24)</f>
+      <c r="C26" s="1">
+        <f>SUM(C2:C25)</f>
+        <v>1092828</v>
+      </c>
+      <c r="D26" s="1">
+        <f>SUM(D2:D25)</f>
         <v>248228</v>
       </c>
-      <c r="E25" s="1">
-        <f>SUM(E2:E24)</f>
-        <v>843300</v>
+      <c r="E26" s="1">
+        <f>SUM(E2:E25)</f>
+        <v>844600</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹1,300.00 by Waheeda (mother) for Arbiya & Didi Sangle
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H25</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -927,7 +927,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1539,34 +1539,60 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v>c3d399da</v>
+      </c>
+      <c r="B24" t="str">
+        <v>985ce939</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Arbiya &amp; Didi Sangle</v>
+      </c>
+      <c r="D24" s="3">
+        <v>46257</v>
+      </c>
+      <c r="E24" s="1">
+        <v>1300</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Waheeda (mother)</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Arbiya &amp; Didi Sangle</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
         <v>de8adadf</v>
       </c>
-      <c r="B24" t="str">
+      <c r="B25" t="str">
         <v>a036f9f7</v>
       </c>
-      <c r="C24" t="str">
+      <c r="C25" t="str">
         <v>Arbiya Bangals</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D25" s="3">
         <v>46263</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E25" s="1">
         <v>550</v>
       </c>
-      <c r="F24" t="str">
+      <c r="F25" t="str">
         <v>Asif Sayyed (Son)</v>
       </c>
-      <c r="G24" t="str">
+      <c r="G25" t="str">
         <v>UPI</v>
       </c>
-      <c r="H24" t="str">
+      <c r="H25" t="str">
         <v>Bangal</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H24"/>
+  <autoFilter ref="A1:H25"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H25"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1687,11 +1713,11 @@
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>1300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2065,11 +2091,11 @@
       </c>
       <c r="D26" s="1">
         <f>SUM(D2:D25)</f>
-        <v>248228</v>
+        <v>249528</v>
       </c>
       <c r="E26" s="1">
         <f>SUM(E2:E25)</f>
-        <v>844600</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update payment: ₹550.00 by Asif Sayyed (Son) for Arbiya Bangals
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -1539,54 +1539,54 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>c3d399da</v>
+        <v>de8adadf</v>
       </c>
       <c r="B24" t="str">
-        <v>985ce939</v>
+        <v>a036f9f7</v>
       </c>
       <c r="C24" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="D24" s="3">
         <v>46257</v>
       </c>
       <c r="E24" s="1">
-        <v>1300</v>
+        <v>550</v>
       </c>
       <c r="F24" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G24" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H24" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Bangal</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>de8adadf</v>
+        <v>c3d399da</v>
       </c>
       <c r="B25" t="str">
-        <v>a036f9f7</v>
+        <v>985ce939</v>
       </c>
       <c r="C25" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
       <c r="D25" s="3">
-        <v>46263</v>
+        <v>46257</v>
       </c>
       <c r="E25" s="1">
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="F25" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G25" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H25" t="str">
-        <v>Bangal</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Invitation Card (treaditional) — ₹3,675.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H25</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -679,248 +679,268 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B14" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C14" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D14" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F14" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B15" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D15" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E15" s="2" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B16" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D16" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E16" s="2" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B17" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D17" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E17" s="2" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B18" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E18" s="2" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B19" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E19" s="2" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B20" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C20" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F20" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B21" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C21" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D21" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F21" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B22" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C22" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D22" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E22" s="2" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B23" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D23" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B24" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C24" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D24" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E24" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F24" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D25" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E25" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F25" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B25" t="str">
+      <c r="B26" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C25" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D25" s="1">
+      <c r="C26" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D26" s="1">
         <v>6190</v>
       </c>
-      <c r="E25" s="2" t="str">
+      <c r="E26" s="2" t="str">
         <v/>
       </c>
-      <c r="F25" t="str">
+      <c r="F26" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F25"/>
+  <autoFilter ref="A1:F26"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F26"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1599,7 +1619,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1855,36 +1875,36 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B14" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C14" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>0</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>0</v>
+        <v>3675</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C15" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -1893,17 +1913,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C16" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -1912,17 +1932,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C17" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -1931,17 +1951,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -1950,17 +1970,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -1969,55 +1989,55 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B20" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B21" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C21" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B22" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C22" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2026,17 +2046,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C23" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2045,62 +2065,81 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B24" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C24" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B25" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C25" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C26" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D26" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E26" s="1">
+        <f>C26-D26</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
         <v>Total</v>
       </c>
-      <c r="C26" s="1">
-        <f>SUM(C2:C25)</f>
-        <v>1092828</v>
-      </c>
-      <c r="D26" s="1">
-        <f>SUM(D2:D25)</f>
+      <c r="C27" s="1">
+        <f>SUM(C2:C26)</f>
+        <v>1096503</v>
+      </c>
+      <c r="D27" s="1">
+        <f>SUM(D2:D26)</f>
         <v>249528</v>
       </c>
-      <c r="E26" s="1">
-        <f>SUM(E2:E25)</f>
-        <v>843300</v>
+      <c r="E27" s="1">
+        <f>SUM(E2:E26)</f>
+        <v>846975</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹3,675.00 by Asif Sayyed (Son) for Invitation Card (treaditional)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H26</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -947,7 +947,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1403,45 +1403,45 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>04a382c3</v>
+        <v>d478d6d7</v>
       </c>
       <c r="B18" t="str">
-        <v>7896f0b1</v>
+        <v>1e95c55a</v>
       </c>
       <c r="C18" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="D18" s="3">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="E18" s="1">
-        <v>24000</v>
+        <v>3675</v>
       </c>
       <c r="F18" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G18" t="str">
-        <v>Debit Card</v>
+        <v>UPI</v>
       </c>
       <c r="H18" t="str">
-        <v>Paid</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>b83ec348</v>
+        <v>04a382c3</v>
       </c>
       <c r="B19" t="str">
-        <v>d5fe8bfd</v>
+        <v>7896f0b1</v>
       </c>
       <c r="C19" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="D19" s="3">
         <v>46257</v>
       </c>
       <c r="E19" s="1">
-        <v>12150</v>
+        <v>24000</v>
       </c>
       <c r="F19" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -1450,128 +1450,128 @@
         <v>Debit Card</v>
       </c>
       <c r="H19" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>965c1bf2</v>
+        <v>b83ec348</v>
       </c>
       <c r="B20" t="str">
-        <v>d1aee56d</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="C20" t="str">
-        <v>Shireen Dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="D20" s="3">
         <v>46257</v>
       </c>
       <c r="E20" s="1">
-        <v>2000</v>
+        <v>12150</v>
       </c>
       <c r="F20" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G20" t="str">
-        <v>UPI</v>
+        <v>Debit Card</v>
       </c>
       <c r="H20" t="str">
-        <v>Shireen Dress paid</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>79903b8b</v>
+        <v>965c1bf2</v>
       </c>
       <c r="B21" t="str">
-        <v>7e3ae131</v>
+        <v>d1aee56d</v>
       </c>
       <c r="C21" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="D21" s="3">
         <v>46257</v>
       </c>
       <c r="E21" s="1">
-        <v>4080</v>
+        <v>2000</v>
       </c>
       <c r="F21" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G21" t="str">
         <v>UPI</v>
       </c>
       <c r="H21" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
+        <v>Shireen Dress paid</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>109c6f27</v>
+        <v>79903b8b</v>
       </c>
       <c r="B22" t="str">
-        <v>4e1fe7bf</v>
+        <v>7e3ae131</v>
       </c>
       <c r="C22" t="str">
-        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
       <c r="D22" s="3">
         <v>46257</v>
       </c>
       <c r="E22" s="1">
-        <v>1000</v>
+        <v>4080</v>
       </c>
       <c r="F22" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G22" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H22" t="str">
-        <v>advance</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>b5b081de</v>
+        <v>109c6f27</v>
       </c>
       <c r="B23" t="str">
-        <v>1bb495b6</v>
+        <v>4e1fe7bf</v>
       </c>
       <c r="C23" t="str">
-        <v>23 Aug Basta lunch at Shahidawat</v>
+        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
       </c>
       <c r="D23" s="3">
         <v>46257</v>
       </c>
       <c r="E23" s="1">
-        <v>2545</v>
+        <v>1000</v>
       </c>
       <c r="F23" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G23" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H23" t="str">
-        <v>23 Aug Basta lunch paid</v>
+        <v>advance</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>de8adadf</v>
+        <v>b5b081de</v>
       </c>
       <c r="B24" t="str">
-        <v>a036f9f7</v>
+        <v>1bb495b6</v>
       </c>
       <c r="C24" t="str">
-        <v>Arbiya Bangals</v>
+        <v>23 Aug Basta lunch at Shahidawat</v>
       </c>
       <c r="D24" s="3">
         <v>46257</v>
       </c>
       <c r="E24" s="1">
-        <v>550</v>
+        <v>2545</v>
       </c>
       <c r="F24" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1580,39 +1580,65 @@
         <v>UPI</v>
       </c>
       <c r="H24" t="str">
-        <v>Bangal</v>
+        <v>23 Aug Basta lunch paid</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>c3d399da</v>
+        <v>de8adadf</v>
       </c>
       <c r="B25" t="str">
-        <v>985ce939</v>
+        <v>a036f9f7</v>
       </c>
       <c r="C25" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="D25" s="3">
         <v>46257</v>
       </c>
       <c r="E25" s="1">
+        <v>550</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G25" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Bangal</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>c3d399da</v>
+      </c>
+      <c r="B26" t="str">
+        <v>985ce939</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Arbiya &amp; Didi Sangle</v>
+      </c>
+      <c r="D26" s="3">
+        <v>46257</v>
+      </c>
+      <c r="E26" s="1">
         <v>1300</v>
       </c>
-      <c r="F25" t="str">
+      <c r="F26" t="str">
         <v>Waheeda (mother)</v>
       </c>
-      <c r="G25" t="str">
+      <c r="G26" t="str">
         <v>Cash</v>
       </c>
-      <c r="H25" t="str">
+      <c r="H26" t="str">
         <v>Arbiya &amp; Didi Sangle</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H25"/>
+  <autoFilter ref="A1:H26"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H26"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1885,11 +1911,11 @@
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>3675</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>3675</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2130,11 +2156,11 @@
       </c>
       <c r="D27" s="1">
         <f>SUM(D2:D26)</f>
-        <v>249528</v>
+        <v>253203</v>
       </c>
       <c r="E27" s="1">
         <f>SUM(E2:E26)</f>
-        <v>846975</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Invitation Card (Shubham) — ₹1,500.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H26</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -679,268 +679,288 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B14" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C14" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D14" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F14" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B15" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C15" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D15" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F15" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B16" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D16" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E16" s="2" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B17" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D17" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E17" s="2" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B18" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E18" s="2" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B19" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E19" s="2" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B20" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E20" s="2" t="str">
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B21" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C21" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D21" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F21" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B22" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C22" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D22" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F22" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B23" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C23" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D23" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B24" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D24" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B25" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C25" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E25" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F25" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D26" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E26" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F26" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B26" t="str">
+      <c r="B27" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C26" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D26" s="1">
+      <c r="C27" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D27" s="1">
         <v>6190</v>
       </c>
-      <c r="E26" s="2" t="str">
+      <c r="E27" s="2" t="str">
         <v/>
       </c>
-      <c r="F26" t="str">
+      <c r="F27" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F26"/>
+  <autoFilter ref="A1:F27"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F27"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1645,7 +1665,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1901,36 +1921,36 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B14" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C14" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>0</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B15" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C15" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -1939,17 +1959,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B16" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C16" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -1958,17 +1978,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C17" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -1977,17 +1997,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -1996,17 +2016,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -2015,17 +2035,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -2034,55 +2054,55 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B21" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C21" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B22" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C22" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B23" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C23" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2091,17 +2111,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C24" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2110,62 +2130,81 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B25" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B26" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C26" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C27" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D27" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E27" s="1">
+        <f>C27-D27</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
         <v>Total</v>
       </c>
-      <c r="C27" s="1">
-        <f>SUM(C2:C26)</f>
-        <v>1096503</v>
-      </c>
-      <c r="D27" s="1">
-        <f>SUM(D2:D26)</f>
+      <c r="C28" s="1">
+        <f>SUM(C2:C27)</f>
+        <v>1098003</v>
+      </c>
+      <c r="D28" s="1">
+        <f>SUM(D2:D27)</f>
         <v>253203</v>
       </c>
-      <c r="E27" s="1">
-        <f>SUM(E2:E26)</f>
-        <v>843300</v>
+      <c r="E28" s="1">
+        <f>SUM(E2:E27)</f>
+        <v>844800</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹1,500.00 by Asif Sayyed (Son) for Invitation Card (Shubham)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H27</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -967,7 +967,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1449,45 +1449,45 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>04a382c3</v>
+        <v>6d30e094</v>
       </c>
       <c r="B19" t="str">
-        <v>7896f0b1</v>
+        <v>aa710190</v>
       </c>
       <c r="C19" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="D19" s="3">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="E19" s="1">
-        <v>24000</v>
+        <v>1500</v>
       </c>
       <c r="F19" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G19" t="str">
-        <v>Debit Card</v>
+        <v>UPI</v>
       </c>
       <c r="H19" t="str">
-        <v>Paid</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>b83ec348</v>
+        <v>04a382c3</v>
       </c>
       <c r="B20" t="str">
-        <v>d5fe8bfd</v>
+        <v>7896f0b1</v>
       </c>
       <c r="C20" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="D20" s="3">
         <v>46257</v>
       </c>
       <c r="E20" s="1">
-        <v>12150</v>
+        <v>24000</v>
       </c>
       <c r="F20" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -1496,128 +1496,128 @@
         <v>Debit Card</v>
       </c>
       <c r="H20" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>965c1bf2</v>
+        <v>b83ec348</v>
       </c>
       <c r="B21" t="str">
-        <v>d1aee56d</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="C21" t="str">
-        <v>Shireen Dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="D21" s="3">
         <v>46257</v>
       </c>
       <c r="E21" s="1">
-        <v>2000</v>
+        <v>12150</v>
       </c>
       <c r="F21" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G21" t="str">
-        <v>UPI</v>
+        <v>Debit Card</v>
       </c>
       <c r="H21" t="str">
-        <v>Shireen Dress paid</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>79903b8b</v>
+        <v>965c1bf2</v>
       </c>
       <c r="B22" t="str">
-        <v>7e3ae131</v>
+        <v>d1aee56d</v>
       </c>
       <c r="C22" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="D22" s="3">
         <v>46257</v>
       </c>
       <c r="E22" s="1">
-        <v>4080</v>
+        <v>2000</v>
       </c>
       <c r="F22" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G22" t="str">
         <v>UPI</v>
       </c>
       <c r="H22" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
+        <v>Shireen Dress paid</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>109c6f27</v>
+        <v>79903b8b</v>
       </c>
       <c r="B23" t="str">
-        <v>4e1fe7bf</v>
+        <v>7e3ae131</v>
       </c>
       <c r="C23" t="str">
-        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
       <c r="D23" s="3">
         <v>46257</v>
       </c>
       <c r="E23" s="1">
-        <v>1000</v>
+        <v>4080</v>
       </c>
       <c r="F23" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G23" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H23" t="str">
-        <v>advance</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>b5b081de</v>
+        <v>109c6f27</v>
       </c>
       <c r="B24" t="str">
-        <v>1bb495b6</v>
+        <v>4e1fe7bf</v>
       </c>
       <c r="C24" t="str">
-        <v>23 Aug Basta lunch at Shahidawat</v>
+        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
       </c>
       <c r="D24" s="3">
         <v>46257</v>
       </c>
       <c r="E24" s="1">
-        <v>2545</v>
+        <v>1000</v>
       </c>
       <c r="F24" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G24" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H24" t="str">
-        <v>23 Aug Basta lunch paid</v>
+        <v>advance</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>de8adadf</v>
+        <v>b5b081de</v>
       </c>
       <c r="B25" t="str">
-        <v>a036f9f7</v>
+        <v>1bb495b6</v>
       </c>
       <c r="C25" t="str">
-        <v>Arbiya Bangals</v>
+        <v>23 Aug Basta lunch at Shahidawat</v>
       </c>
       <c r="D25" s="3">
         <v>46257</v>
       </c>
       <c r="E25" s="1">
-        <v>550</v>
+        <v>2545</v>
       </c>
       <c r="F25" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1626,39 +1626,65 @@
         <v>UPI</v>
       </c>
       <c r="H25" t="str">
-        <v>Bangal</v>
+        <v>23 Aug Basta lunch paid</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>c3d399da</v>
+        <v>de8adadf</v>
       </c>
       <c r="B26" t="str">
-        <v>985ce939</v>
+        <v>a036f9f7</v>
       </c>
       <c r="C26" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="D26" s="3">
         <v>46257</v>
       </c>
       <c r="E26" s="1">
+        <v>550</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G26" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Bangal</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>c3d399da</v>
+      </c>
+      <c r="B27" t="str">
+        <v>985ce939</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Arbiya &amp; Didi Sangle</v>
+      </c>
+      <c r="D27" s="3">
+        <v>46257</v>
+      </c>
+      <c r="E27" s="1">
         <v>1300</v>
       </c>
-      <c r="F26" t="str">
+      <c r="F27" t="str">
         <v>Waheeda (mother)</v>
       </c>
-      <c r="G26" t="str">
+      <c r="G27" t="str">
         <v>Cash</v>
       </c>
-      <c r="H26" t="str">
+      <c r="H27" t="str">
         <v>Arbiya &amp; Didi Sangle</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H26"/>
+  <autoFilter ref="A1:H27"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1931,11 +1957,11 @@
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2195,11 +2221,11 @@
       </c>
       <c r="D28" s="1">
         <f>SUM(D2:D27)</f>
-        <v>253203</v>
+        <v>254703</v>
       </c>
       <c r="E28" s="1">
         <f>SUM(E2:E27)</f>
-        <v>844800</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Bari ka saman — ₹2,200.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H27</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -559,408 +559,428 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>631875ca</v>
+        <v>0e8bf89b</v>
       </c>
       <c r="B8" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="C8" t="str">
-        <v>Decoration</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D8" s="1">
-        <v>143000</v>
+        <v>2200</v>
       </c>
       <c r="E8" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>Hall decoration</v>
+        <v>Bari ka saman</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B9" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C9" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D9" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E9" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F9" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B10" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D10" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E10" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F10" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B11" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C11" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D11" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E11" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F11" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B12" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C12" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D12" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E12" s="2" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B13" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C13" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D13" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E13" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F13" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>aa710190</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B14" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C14" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D14" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v>7385125161</v>
+        <v>9226111899</v>
       </c>
       <c r="F14" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B15" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C15" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D15" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F15" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B16" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C16" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D16" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F16" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B17" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D17" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E17" s="2" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B18" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E18" s="2" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B19" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E19" s="2" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>113a1c1a</v>
+        <v>a78dd739</v>
       </c>
       <c r="B20" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E20" s="2" t="str">
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>bride 3 dress</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B21" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D21" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E21" s="2" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B22" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C22" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D22" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E22" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F22" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B23" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C23" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D23" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F23" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B24" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C24" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D24" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B25" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B26" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C26" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D26" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E26" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F26" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D27" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E27" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F27" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B27" t="str">
+      <c r="B28" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C27" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D27" s="1">
+      <c r="C28" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D28" s="1">
         <v>6190</v>
       </c>
-      <c r="E27" s="2" t="str">
+      <c r="E28" s="2" t="str">
         <v/>
       </c>
-      <c r="F27" t="str">
+      <c r="F28" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F27"/>
+  <autoFilter ref="A1:F28"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1691,7 +1711,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1833,55 +1853,55 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="B8" t="str">
-        <v>Decoration</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C8" s="1">
-        <v>143000</v>
+        <v>2200</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
-        <v>128000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B9" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C9" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B10" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C10" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -1890,17 +1910,17 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B11" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C11" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -1909,17 +1929,17 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B12" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C12" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
@@ -1928,55 +1948,55 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B13" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C13" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B14" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C14" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>50000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B15" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C15" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -1985,17 +2005,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B16" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C16" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -2004,17 +2024,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B17" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C17" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -2023,17 +2043,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -2042,17 +2062,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -2061,17 +2081,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>400</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -2080,17 +2100,17 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C21" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -2099,55 +2119,55 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B22" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C22" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B23" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C23" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B24" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C24" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2156,17 +2176,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -2175,62 +2195,81 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B26" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C26" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B27" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C27" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C28" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D28" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E28" s="1">
+        <f>C28-D28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>Total</v>
       </c>
-      <c r="C28" s="1">
-        <f>SUM(C2:C27)</f>
-        <v>1098003</v>
-      </c>
-      <c r="D28" s="1">
-        <f>SUM(D2:D27)</f>
+      <c r="C29" s="1">
+        <f>SUM(C2:C28)</f>
+        <v>1100203</v>
+      </c>
+      <c r="D29" s="1">
+        <f>SUM(D2:D28)</f>
         <v>254703</v>
       </c>
-      <c r="E28" s="1">
-        <f>SUM(E2:E27)</f>
-        <v>843300</v>
+      <c r="E29" s="1">
+        <f>SUM(E2:E28)</f>
+        <v>845500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹2,200.00 by Umar Sayyed (Father) for Bari ka saman
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H28</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -987,7 +987,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1701,10 +1701,36 @@
         <v>Arbiya &amp; Didi Sangle</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>dccde075</v>
+      </c>
+      <c r="B28" t="str">
+        <v>0e8bf89b</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Bari ka saman</v>
+      </c>
+      <c r="D28" s="3">
+        <v>46259</v>
+      </c>
+      <c r="E28" s="1">
+        <v>2200</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H28" t="str">
+        <v>paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H27"/>
+  <autoFilter ref="A1:H28"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1863,11 +1889,11 @@
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
-        <v>2200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2260,11 +2286,11 @@
       </c>
       <c r="D29" s="1">
         <f>SUM(D2:D28)</f>
-        <v>254703</v>
+        <v>256903</v>
       </c>
       <c r="E29" s="1">
         <f>SUM(E2:E28)</f>
-        <v>845500</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Navkar Sales Corporation — ₹8,649.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H28</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -819,168 +819,188 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>113a1c1a</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B21" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C21" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D21" s="1">
-        <v>5700</v>
+        <v>8649</v>
       </c>
       <c r="E21" s="2" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>bride 3 dress</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B22" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D22" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E22" s="2" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B23" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C23" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D23" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E23" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F23" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B24" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C24" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D24" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E24" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F24" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B25" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C25" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D25" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B26" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D26" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B27" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C27" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D27" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E27" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F27" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
+        <v>04ece648</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Soyarik mangal karyalay</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Venue &amp; Hall</v>
+      </c>
+      <c r="D28" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E28" s="2" t="str">
+        <v>9850444117</v>
+      </c>
+      <c r="F28" t="str">
+        <v>venue for reception</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>bd5f8d26</v>
       </c>
-      <c r="B28" t="str">
+      <c r="B29" t="str">
         <v>Star Bazaar - Prewedding dress</v>
       </c>
-      <c r="C28" t="str">
-        <v>Clothing &amp; Jewellery</v>
-      </c>
-      <c r="D28" s="1">
+      <c r="C29" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D29" s="1">
         <v>6190</v>
       </c>
-      <c r="E28" s="2" t="str">
+      <c r="E29" s="2" t="str">
         <v/>
       </c>
-      <c r="F28" t="str">
+      <c r="F29" t="str">
         <v>Prewedding dress</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F28"/>
+  <autoFilter ref="A1:F29"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1737,7 +1757,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2126,36 +2146,36 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B21" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C21" s="1">
-        <v>5700</v>
+        <v>8649</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>0</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>0</v>
+        <v>8649</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C22" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2164,55 +2184,55 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B23" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C23" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B24" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C24" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B25" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C25" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -2221,17 +2241,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C26" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -2240,62 +2260,81 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B27" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C27" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B28" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C28" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="C29" s="1">
+        <v>6190</v>
+      </c>
+      <c r="D29" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
+        <v>6190</v>
+      </c>
+      <c r="E29" s="1">
+        <f>C29-D29</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
         <v>Total</v>
       </c>
-      <c r="C29" s="1">
-        <f>SUM(C2:C28)</f>
-        <v>1100203</v>
-      </c>
-      <c r="D29" s="1">
-        <f>SUM(D2:D28)</f>
+      <c r="C30" s="1">
+        <f>SUM(C2:C29)</f>
+        <v>1108852</v>
+      </c>
+      <c r="D30" s="1">
+        <f>SUM(D2:D29)</f>
         <v>256903</v>
       </c>
-      <c r="E29" s="1">
-        <f>SUM(E2:E28)</f>
-        <v>843300</v>
+      <c r="E30" s="1">
+        <f>SUM(E2:E29)</f>
+        <v>851949</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹8,649.00 by Asif Sayyed (Son) for Navkar Sales Corporation
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H29</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1007,7 +1007,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1747,10 +1747,36 @@
         <v>paid</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>bbfbed2b</v>
+      </c>
+      <c r="B29" t="str">
+        <v>eebc3aaf</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Navkar Sales Corporation</v>
+      </c>
+      <c r="D29" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E29" s="1">
+        <v>8649</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G29" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H29" t="str">
+        <v>paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H28"/>
+  <autoFilter ref="A1:H29"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2156,11 +2182,11 @@
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>8649</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
-        <v>8649</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -2325,11 +2351,11 @@
       </c>
       <c r="D30" s="1">
         <f>SUM(D2:D29)</f>
-        <v>256903</v>
+        <v>265552</v>
       </c>
       <c r="E30" s="1">
         <f>SUM(E2:E29)</f>
-        <v>851949</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Tushar Traders Oil — ₹5,100.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H29</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -997,10 +997,30 @@
         <v>Prewedding dress</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D30" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E30" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F29"/>
+  <autoFilter ref="A1:F30"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F30"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1783,7 +1803,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2343,24 +2363,43 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C30" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D30" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="1">
+        <f>C30-D30</f>
+        <v>5100</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
         <v>Total</v>
       </c>
-      <c r="C30" s="1">
-        <f>SUM(C2:C29)</f>
-        <v>1108852</v>
-      </c>
-      <c r="D30" s="1">
-        <f>SUM(D2:D29)</f>
+      <c r="C31" s="1">
+        <f>SUM(C2:C30)</f>
+        <v>1113952</v>
+      </c>
+      <c r="D31" s="1">
+        <f>SUM(D2:D30)</f>
         <v>265552</v>
       </c>
-      <c r="E30" s="1">
-        <f>SUM(E2:E29)</f>
-        <v>843300</v>
+      <c r="E31" s="1">
+        <f>SUM(E2:E30)</f>
+        <v>848400</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹5,100.00 by Asif Sayyed (Son) for Tushar Traders Oil
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H30</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1027,7 +1027,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1793,10 +1793,36 @@
         <v>paid</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>c9cf6d4a</v>
+      </c>
+      <c r="B30" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="D30" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E30" s="1">
+        <v>5100</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G30" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H30" t="str">
+        <v>paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H29"/>
+  <autoFilter ref="A1:H30"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H30"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2373,11 +2399,11 @@
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>5100</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
-        <v>5100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -2390,11 +2416,11 @@
       </c>
       <c r="D31" s="1">
         <f>SUM(D2:D30)</f>
-        <v>265552</v>
+        <v>270652</v>
       </c>
       <c r="E31" s="1">
         <f>SUM(E2:E30)</f>
-        <v>848400</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Bhavesh Treaders (kirana) — ₹4,600.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H30</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -579,448 +579,468 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>631875ca</v>
+        <v>0beedebe</v>
       </c>
       <c r="B9" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="C9" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D9" s="1">
-        <v>143000</v>
+        <v>4600</v>
       </c>
       <c r="E9" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F9" t="str">
-        <v>Hall decoration</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B10" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C10" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D10" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E10" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F10" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B11" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D11" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E11" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F11" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B12" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C12" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D12" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F12" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B13" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C13" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D13" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E13" s="2" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B14" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C14" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D14" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F14" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>aa710190</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B15" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C15" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D15" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v>7385125161</v>
+        <v>9226111899</v>
       </c>
       <c r="F15" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B16" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C16" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D16" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F16" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B17" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C17" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D17" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F17" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B18" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D18" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E18" s="2" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B19" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E19" s="2" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B20" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E20" s="2" t="str">
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>eebc3aaf</v>
+        <v>a78dd739</v>
       </c>
       <c r="B21" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C21" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D21" s="1">
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="E21" s="2" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>113a1c1a</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B22" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C22" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D22" s="1">
-        <v>5700</v>
+        <v>8649</v>
       </c>
       <c r="E22" s="2" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>bride 3 dress</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B23" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D23" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B24" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C24" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D24" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E24" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F24" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B25" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C25" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D25" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E25" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F25" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B26" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C26" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D26" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B27" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D27" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B28" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C28" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D28" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E28" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F28" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B29" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D29" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E29" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F29" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B30" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C30" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B31" t="str">
         <v>Tushar Traders Oil</v>
       </c>
+      <c r="C31" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D31" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E31" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F30"/>
+  <autoFilter ref="A1:F31"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F31"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1829,7 +1849,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1990,55 +2010,55 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="B9" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C9" s="1">
-        <v>143000</v>
+        <v>4600</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>128000</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B10" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C10" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B11" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C11" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -2047,17 +2067,17 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B12" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C12" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
@@ -2066,17 +2086,17 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B13" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C13" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -2085,55 +2105,55 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B14" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C14" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B15" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C15" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>50000</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B16" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C16" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -2142,17 +2162,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B17" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C17" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -2161,17 +2181,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B18" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C18" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -2180,17 +2200,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -2199,17 +2219,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -2218,17 +2238,17 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B21" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C21" s="1">
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -2237,17 +2257,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B22" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C22" s="1">
-        <v>5700</v>
+        <v>8649</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>8649</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2256,17 +2276,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C23" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2275,55 +2295,55 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B24" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C24" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B25" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C25" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B26" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C26" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -2332,17 +2352,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C27" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -2351,55 +2371,55 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B28" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C28" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C29" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B30" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -2408,24 +2428,43 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C31" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D31" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E31" s="1">
+        <f>C31-D31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
         <v>Total</v>
       </c>
-      <c r="C31" s="1">
-        <f>SUM(C2:C30)</f>
-        <v>1113952</v>
-      </c>
-      <c r="D31" s="1">
-        <f>SUM(D2:D30)</f>
+      <c r="C32" s="1">
+        <f>SUM(C2:C31)</f>
+        <v>1118552</v>
+      </c>
+      <c r="D32" s="1">
+        <f>SUM(D2:D31)</f>
         <v>270652</v>
       </c>
-      <c r="E31" s="1">
-        <f>SUM(E2:E30)</f>
-        <v>843300</v>
+      <c r="E32" s="1">
+        <f>SUM(E2:E31)</f>
+        <v>847900</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹4,600.00 by Asif Sayyed (Son) for Bhavesh Treaders (kirana)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H31</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1047,7 +1047,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1839,10 +1839,36 @@
         <v>paid</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>9c9ac50b</v>
+      </c>
+      <c r="B31" t="str">
+        <v>0beedebe</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Bhavesh Treaders (kirana)</v>
+      </c>
+      <c r="D31" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E31" s="1">
+        <v>4600</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G31" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Bhavesh Treaders (kirana) paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H30"/>
+  <autoFilter ref="A1:H31"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H31"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2020,11 +2046,11 @@
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>4600</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>4600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2455,11 +2481,11 @@
       </c>
       <c r="D32" s="1">
         <f>SUM(D2:D31)</f>
-        <v>270652</v>
+        <v>275252</v>
       </c>
       <c r="E32" s="1">
         <f>SUM(E2:E31)</f>
-        <v>847900</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: New Balaji Treaders — ₹575.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H31</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -859,188 +859,208 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B23" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C23" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D23" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B24" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D24" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B25" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C25" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E25" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F25" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>6d180155</v>
+        <v>beb44857</v>
       </c>
       <c r="B26" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C26" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D26" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="E26" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F26" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B27" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C27" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D27" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B28" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D28" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B29" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C29" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D29" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E29" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F29" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B30" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D30" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E30" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F30" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B31" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C31" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B32" t="str">
         <v>Tushar Traders Oil</v>
       </c>
+      <c r="C32" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D32" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F31"/>
+  <autoFilter ref="A1:F32"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F32"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1875,7 +1895,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2302,36 +2322,36 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B23" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C23" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>0</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
-        <v>0</v>
+        <v>575</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C24" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2340,55 +2360,55 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B25" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B26" t="str">
-        <v>Miscellaneous</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C26" s="1">
-        <v>11840</v>
+        <v>100000</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>10000</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B27" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C27" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -2397,17 +2417,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C28" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -2416,55 +2436,55 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B29" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C29" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C30" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B31" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -2473,24 +2493,43 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C32" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D32" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E32" s="1">
+        <f>C32-D32</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
         <v>Total</v>
       </c>
-      <c r="C32" s="1">
-        <f>SUM(C2:C31)</f>
-        <v>1118552</v>
-      </c>
-      <c r="D32" s="1">
-        <f>SUM(D2:D31)</f>
+      <c r="C33" s="1">
+        <f>SUM(C2:C32)</f>
+        <v>1119127</v>
+      </c>
+      <c r="D33" s="1">
+        <f>SUM(D2:D32)</f>
         <v>275252</v>
       </c>
-      <c r="E32" s="1">
-        <f>SUM(E2:E31)</f>
-        <v>843300</v>
+      <c r="E33" s="1">
+        <f>SUM(E2:E32)</f>
+        <v>843875</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E33"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹575.00 by Asif Sayyed (Son) for New Balaji Treaders
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H32</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1067,7 +1067,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1885,10 +1885,36 @@
         <v>Bhavesh Treaders (kirana) paid</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>cda2807c</v>
+      </c>
+      <c r="B32" t="str">
+        <v>e6b755dc</v>
+      </c>
+      <c r="C32" t="str">
+        <v>New Balaji Treaders</v>
+      </c>
+      <c r="D32" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E32" s="1">
+        <v>575</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G32" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H32" t="str">
+        <v>paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H31"/>
+  <autoFilter ref="A1:H32"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H32"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2332,11 +2358,11 @@
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>575</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
-        <v>575</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -2520,11 +2546,11 @@
       </c>
       <c r="D33" s="1">
         <f>SUM(D2:D32)</f>
-        <v>275252</v>
+        <v>275827</v>
       </c>
       <c r="E33" s="1">
         <f>SUM(E2:E32)</f>
-        <v>843875</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Pravin Masale — ₹3,345.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H32</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -939,128 +939,148 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B27" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C27" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D27" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B28" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C28" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D28" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B29" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D29" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B30" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C30" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E30" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F30" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B31" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D31" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E31" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F31" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B32" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C32" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B33" t="str">
         <v>Tushar Traders Oil</v>
       </c>
+      <c r="C33" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D33" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F32"/>
+  <autoFilter ref="A1:F33"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F33"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1921,7 +1941,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2424,36 +2444,36 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B27" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C27" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>0</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
-        <v>0</v>
+        <v>3345</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B28" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C28" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -2462,17 +2482,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C29" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -2481,55 +2501,55 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B30" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C31" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B32" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -2538,24 +2558,43 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C33" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D33" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E33" s="1">
+        <f>C33-D33</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
         <v>Total</v>
       </c>
-      <c r="C33" s="1">
-        <f>SUM(C2:C32)</f>
-        <v>1119127</v>
-      </c>
-      <c r="D33" s="1">
-        <f>SUM(D2:D32)</f>
+      <c r="C34" s="1">
+        <f>SUM(C2:C33)</f>
+        <v>1122472</v>
+      </c>
+      <c r="D34" s="1">
+        <f>SUM(D2:D33)</f>
         <v>275827</v>
       </c>
-      <c r="E33" s="1">
-        <f>SUM(E2:E32)</f>
-        <v>843300</v>
+      <c r="E34" s="1">
+        <f>SUM(E2:E33)</f>
+        <v>846645</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹3,345.00 by Asif Sayyed (Son) for Pravin Masale
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H33</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1087,7 +1087,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1931,10 +1931,36 @@
         <v>paid</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>62d1ce54</v>
+      </c>
+      <c r="B33" t="str">
+        <v>89c1b231</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Pravin Masale</v>
+      </c>
+      <c r="D33" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E33" s="1">
+        <v>3345</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G33" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Pravin Masal Paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H32"/>
+  <autoFilter ref="A1:H33"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H33"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2454,11 +2480,11 @@
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>3345</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
-        <v>3345</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -2585,11 +2611,11 @@
       </c>
       <c r="D34" s="1">
         <f>SUM(D2:D33)</f>
-        <v>275827</v>
+        <v>279172</v>
       </c>
       <c r="E34" s="1">
         <f>SUM(E2:E33)</f>
-        <v>846645</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Bhavesh Treaders (karele & javas) — ₹270.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H33</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -579,508 +579,528 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>0beedebe</v>
+        <v>1aa31869</v>
       </c>
       <c r="B9" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="C9" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D9" s="1">
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="E9" s="2" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>631875ca</v>
+        <v>0beedebe</v>
       </c>
       <c r="B10" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="C10" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D10" s="1">
-        <v>143000</v>
+        <v>4600</v>
       </c>
       <c r="E10" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F10" t="str">
-        <v>Hall decoration</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B11" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C11" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D11" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E11" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F11" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B12" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D12" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F12" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B13" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C13" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D13" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E13" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F13" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B14" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C14" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D14" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E14" s="2" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B15" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C15" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D15" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F15" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>aa710190</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B16" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C16" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D16" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v>7385125161</v>
+        <v>9226111899</v>
       </c>
       <c r="F16" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B17" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C17" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D17" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F17" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B18" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C18" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D18" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F18" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B19" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D19" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E19" s="2" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B20" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E20" s="2" t="str">
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B21" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D21" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E21" s="2" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>eebc3aaf</v>
+        <v>a78dd739</v>
       </c>
       <c r="B22" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C22" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D22" s="1">
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="E22" s="2" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B23" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C23" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D23" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B24" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C24" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D24" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B25" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B26" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C26" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D26" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E26" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F26" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B27" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C27" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D27" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E27" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F27" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B28" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C28" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D28" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B29" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D29" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B30" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B31" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C31" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E31" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F31" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B32" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D32" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E32" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F32" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B33" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C33" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B34" t="str">
         <v>Tushar Traders Oil</v>
       </c>
+      <c r="C34" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D34" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E34" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F33"/>
+  <autoFilter ref="A1:F34"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1967,7 +1987,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2128,74 +2148,74 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="B9" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C9" s="1">
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>4600</v>
+        <v>0</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>0</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="B10" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C10" s="1">
-        <v>143000</v>
+        <v>4600</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>4600</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
-        <v>128000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B11" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C11" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B12" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C12" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
@@ -2204,17 +2224,17 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B13" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C13" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -2223,17 +2243,17 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B14" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C14" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -2242,55 +2262,55 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B15" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C15" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B16" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C16" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>50000</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B17" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C17" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -2299,17 +2319,17 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B18" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C18" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -2318,17 +2338,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B19" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C19" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -2337,17 +2357,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -2356,17 +2376,17 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C21" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -2375,17 +2395,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B22" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C22" s="1">
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2394,17 +2414,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B23" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C23" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2413,17 +2433,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B24" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C24" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2432,17 +2452,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -2451,55 +2471,55 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B26" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C26" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B27" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C27" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>10000</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B28" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C28" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -2508,17 +2528,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B29" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C29" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -2527,17 +2547,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B30" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -2546,55 +2566,55 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B31" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C32" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B33" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -2603,24 +2623,43 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C34" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D34" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E34" s="1">
+        <f>C34-D34</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
         <v>Total</v>
       </c>
-      <c r="C34" s="1">
-        <f>SUM(C2:C33)</f>
-        <v>1122472</v>
-      </c>
-      <c r="D34" s="1">
-        <f>SUM(D2:D33)</f>
+      <c r="C35" s="1">
+        <f>SUM(C2:C34)</f>
+        <v>1122742</v>
+      </c>
+      <c r="D35" s="1">
+        <f>SUM(D2:D34)</f>
         <v>279172</v>
       </c>
-      <c r="E34" s="1">
-        <f>SUM(E2:E33)</f>
-        <v>843300</v>
+      <c r="E35" s="1">
+        <f>SUM(E2:E34)</f>
+        <v>843570</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹270.00 by Waheeda (mother) for Bhavesh Treaders (karele & javas)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H34</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1107,7 +1107,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1977,10 +1977,36 @@
         <v>Pravin Masal Paid</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>13ce4f28</v>
+      </c>
+      <c r="B34" t="str">
+        <v>1aa31869</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
+      </c>
+      <c r="D34" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E34" s="1">
+        <v>270</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Waheeda (mother)</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H33"/>
+  <autoFilter ref="A1:H34"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2158,11 +2184,11 @@
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>270</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
-        <v>270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2650,11 +2676,11 @@
       </c>
       <c r="D35" s="1">
         <f>SUM(D2:D34)</f>
-        <v>279172</v>
+        <v>279442</v>
       </c>
       <c r="E35" s="1">
         <f>SUM(E2:E34)</f>
-        <v>843570</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Cream House Lunch — ₹1,124.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H34</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -619,488 +619,508 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>631875ca</v>
+        <v>05d27deb</v>
       </c>
       <c r="B11" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="C11" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D11" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="E11" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F11" t="str">
-        <v>Hall decoration</v>
+        <v>Cream House Lunch</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B12" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C12" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D12" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F12" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B13" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D13" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E13" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F13" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B14" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C14" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D14" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F14" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B15" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C15" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D15" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E15" s="2" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B16" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C16" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D16" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>aa710190</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B17" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C17" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D17" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v>7385125161</v>
+        <v>9226111899</v>
       </c>
       <c r="F17" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B18" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C18" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D18" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F18" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B19" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C19" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D19" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F19" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B20" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D20" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E20" s="2" t="str">
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B21" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D21" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E21" s="2" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B22" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D22" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E22" s="2" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>eebc3aaf</v>
+        <v>a78dd739</v>
       </c>
       <c r="B23" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C23" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D23" s="1">
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B24" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C24" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D24" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B25" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C25" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D25" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B26" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D26" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>beb44857</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B27" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C27" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D27" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="E27" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F27" t="str">
-        <v>Photography cost</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B28" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C28" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D28" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E28" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F28" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B29" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C29" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D29" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B30" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D30" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B31" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D31" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B32" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C32" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E32" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F32" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B33" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D33" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E33" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F33" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B34" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C34" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B35" t="str">
         <v>Tushar Traders Oil</v>
       </c>
+      <c r="C35" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D35" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E35" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F34"/>
+  <autoFilter ref="A1:F35"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2013,7 +2033,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2212,55 +2232,55 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="B11" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C11" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
-        <v>128000</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B12" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C12" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B13" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C13" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
@@ -2269,17 +2289,17 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B14" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C14" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -2288,17 +2308,17 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B15" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C15" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -2307,55 +2327,55 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B16" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C16" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B17" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C17" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>50000</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B18" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C18" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
@@ -2364,17 +2384,17 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B19" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C19" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -2383,17 +2403,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B20" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C20" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -2402,17 +2422,17 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C21" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -2421,17 +2441,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C22" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2440,17 +2460,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B23" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C23" s="1">
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2459,17 +2479,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B24" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C24" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2478,17 +2498,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B25" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C25" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -2497,17 +2517,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B26" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C26" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -2516,55 +2536,55 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B27" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C27" s="1">
-        <v>100000</v>
+        <v>24000</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>24000</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B28" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C28" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>10000</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B29" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C29" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -2573,17 +2593,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B30" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C30" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -2592,17 +2612,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B31" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C31" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -2611,55 +2631,55 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B32" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C33" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B34" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -2668,24 +2688,43 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C35" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D35" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E35" s="1">
+        <f>C35-D35</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
         <v>Total</v>
       </c>
-      <c r="C35" s="1">
-        <f>SUM(C2:C34)</f>
-        <v>1122742</v>
-      </c>
-      <c r="D35" s="1">
-        <f>SUM(D2:D34)</f>
+      <c r="C36" s="1">
+        <f>SUM(C2:C35)</f>
+        <v>1123866</v>
+      </c>
+      <c r="D36" s="1">
+        <f>SUM(D2:D35)</f>
         <v>279442</v>
       </c>
-      <c r="E35" s="1">
-        <f>SUM(E2:E34)</f>
-        <v>843300</v>
+      <c r="E36" s="1">
+        <f>SUM(E2:E35)</f>
+        <v>844424</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹1,124.00 by Asif Sayyed (Son) for Cream House Lunch
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H35</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1127,7 +1127,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2023,10 +2023,36 @@
         <v/>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>c2ac5cbf</v>
+      </c>
+      <c r="B35" t="str">
+        <v>05d27deb</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Cream House Lunch</v>
+      </c>
+      <c r="D35" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E35" s="1">
+        <v>1124</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G35" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Cream House Lunch paid</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H34"/>
+  <autoFilter ref="A1:H35"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2242,11 +2268,11 @@
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>1124</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
-        <v>1124</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2715,11 +2741,11 @@
       </c>
       <c r="D36" s="1">
         <f>SUM(D2:D35)</f>
-        <v>279442</v>
+        <v>280566</v>
       </c>
       <c r="E36" s="1">
         <f>SUM(E2:E35)</f>
-        <v>844424</v>
+        <v>843300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record payment: ₹10,000.00 by Asif Sayyed (Son) for Pratap films and Photography
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H36</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1127,7 +1127,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2049,10 +2049,36 @@
         <v>Cream House Lunch paid</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>a7faa1c7</v>
+      </c>
+      <c r="B36" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="D36" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E36" s="1">
+        <v>10000</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G36" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H36" t="str">
+        <v>second installment</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H35"/>
+  <autoFilter ref="A1:H36"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2591,11 +2617,11 @@
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
-        <v>90000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="29">
@@ -2741,11 +2767,11 @@
       </c>
       <c r="D36" s="1">
         <f>SUM(D2:D35)</f>
-        <v>280566</v>
+        <v>290566</v>
       </c>
       <c r="E36" s="1">
         <f>SUM(E2:E35)</f>
-        <v>843300</v>
+        <v>833300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Petrol Glanza — ₹4,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H36</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -959,168 +959,188 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>beb44857</v>
+        <v>0421ab42</v>
       </c>
       <c r="B28" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C28" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D28" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E28" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F28" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B29" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C29" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D29" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E29" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F29" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B30" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C30" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D30" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>18d2728f</v>
+        <v>6d180155</v>
       </c>
       <c r="B31" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D31" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Baste k sadiya</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>d1aee56d</v>
+        <v>18d2728f</v>
       </c>
       <c r="B32" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="C32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Shireen Dress</v>
+        <v>Baste k sadiya</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B33" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C33" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E33" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F33" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B34" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D34" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E34" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F34" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B35" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C35" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B36" t="str">
         <v>Tushar Traders Oil</v>
       </c>
+      <c r="C36" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D36" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E36" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F35"/>
+  <autoFilter ref="A1:F36"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2085,7 +2105,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2607,55 +2627,55 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B28" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C28" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
-        <v>80000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B29" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C29" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>20000</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
-        <v>0</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B30" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C30" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -2664,17 +2684,17 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Sadi basta</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B31" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C31" s="1">
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>11840</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -2683,17 +2703,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Shireen Dress</v>
+        <v>Sadi basta</v>
       </c>
       <c r="B32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -2702,55 +2722,55 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B33" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C34" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B35" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -2759,24 +2779,43 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C36" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D36" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E36" s="1">
+        <f>C36-D36</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
         <v>Total</v>
       </c>
-      <c r="C36" s="1">
-        <f>SUM(C2:C35)</f>
-        <v>1123866</v>
-      </c>
-      <c r="D36" s="1">
-        <f>SUM(D2:D35)</f>
+      <c r="C37" s="1">
+        <f>SUM(C2:C36)</f>
+        <v>1127866</v>
+      </c>
+      <c r="D37" s="1">
+        <f>SUM(D2:D36)</f>
         <v>290566</v>
       </c>
-      <c r="E36" s="1">
-        <f>SUM(E2:E35)</f>
-        <v>833300</v>
+      <c r="E37" s="1">
+        <f>SUM(E2:E36)</f>
+        <v>837300</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹4,000.00 by Umar Sayyed (Father) for Petrol Glanza
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H37</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1147,7 +1147,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1889,45 +1889,45 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>bbfbed2b</v>
+        <v>3c9c77ed</v>
       </c>
       <c r="B29" t="str">
-        <v>eebc3aaf</v>
+        <v>0421ab42</v>
       </c>
       <c r="C29" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="D29" s="3">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="E29" s="1">
-        <v>8649</v>
+        <v>4000</v>
       </c>
       <c r="F29" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G29" t="str">
-        <v>UPI</v>
+        <v>Debit Card</v>
       </c>
       <c r="H29" t="str">
-        <v>paid</v>
+        <v>Petrol Paid</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>c9cf6d4a</v>
+        <v>bbfbed2b</v>
       </c>
       <c r="B30" t="str">
-        <v>db4969e8</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="C30" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="D30" s="3">
         <v>46263</v>
       </c>
       <c r="E30" s="1">
-        <v>5100</v>
+        <v>8649</v>
       </c>
       <c r="F30" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1941,19 +1941,19 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>9c9ac50b</v>
+        <v>c9cf6d4a</v>
       </c>
       <c r="B31" t="str">
-        <v>0beedebe</v>
+        <v>db4969e8</v>
       </c>
       <c r="C31" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="D31" s="3">
         <v>46263</v>
       </c>
       <c r="E31" s="1">
-        <v>4600</v>
+        <v>5100</v>
       </c>
       <c r="F31" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1962,24 +1962,24 @@
         <v>UPI</v>
       </c>
       <c r="H31" t="str">
-        <v>Bhavesh Treaders (kirana) paid</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>cda2807c</v>
+        <v>9c9ac50b</v>
       </c>
       <c r="B32" t="str">
-        <v>e6b755dc</v>
+        <v>0beedebe</v>
       </c>
       <c r="C32" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="D32" s="3">
         <v>46263</v>
       </c>
       <c r="E32" s="1">
-        <v>575</v>
+        <v>4600</v>
       </c>
       <c r="F32" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1988,24 +1988,24 @@
         <v>UPI</v>
       </c>
       <c r="H32" t="str">
-        <v>paid</v>
+        <v>Bhavesh Treaders (kirana) paid</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>62d1ce54</v>
+        <v>cda2807c</v>
       </c>
       <c r="B33" t="str">
-        <v>89c1b231</v>
+        <v>e6b755dc</v>
       </c>
       <c r="C33" t="str">
-        <v>Pravin Masale</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="D33" s="3">
         <v>46263</v>
       </c>
       <c r="E33" s="1">
-        <v>3345</v>
+        <v>575</v>
       </c>
       <c r="F33" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2014,76 +2014,76 @@
         <v>UPI</v>
       </c>
       <c r="H33" t="str">
-        <v>Pravin Masal Paid</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>13ce4f28</v>
+        <v>62d1ce54</v>
       </c>
       <c r="B34" t="str">
-        <v>1aa31869</v>
+        <v>89c1b231</v>
       </c>
       <c r="C34" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="D34" s="3">
         <v>46263</v>
       </c>
       <c r="E34" s="1">
-        <v>270</v>
+        <v>3345</v>
       </c>
       <c r="F34" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G34" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>Pravin Masal Paid</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>c2ac5cbf</v>
+        <v>13ce4f28</v>
       </c>
       <c r="B35" t="str">
-        <v>05d27deb</v>
+        <v>1aa31869</v>
       </c>
       <c r="C35" t="str">
-        <v>Cream House Lunch</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="D35" s="3">
         <v>46263</v>
       </c>
       <c r="E35" s="1">
-        <v>1124</v>
+        <v>270</v>
       </c>
       <c r="F35" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G35" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H35" t="str">
-        <v>Cream House Lunch paid</v>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>a7faa1c7</v>
+        <v>c2ac5cbf</v>
       </c>
       <c r="B36" t="str">
-        <v>beb44857</v>
+        <v>05d27deb</v>
       </c>
       <c r="C36" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="D36" s="3">
         <v>46263</v>
       </c>
       <c r="E36" s="1">
-        <v>10000</v>
+        <v>1124</v>
       </c>
       <c r="F36" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2092,13 +2092,39 @@
         <v>UPI</v>
       </c>
       <c r="H36" t="str">
+        <v>Cream House Lunch paid</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>a7faa1c7</v>
+      </c>
+      <c r="B37" t="str">
+        <v>beb44857</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Pratap films and Photography</v>
+      </c>
+      <c r="D37" s="3">
+        <v>46263</v>
+      </c>
+      <c r="E37" s="1">
+        <v>10000</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G37" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H37" t="str">
         <v>second installment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H36"/>
+  <autoFilter ref="A1:H37"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2637,11 +2663,11 @@
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
-        <v>4000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -2806,11 +2832,11 @@
       </c>
       <c r="D37" s="1">
         <f>SUM(D2:D36)</f>
-        <v>290566</v>
+        <v>294566</v>
       </c>
       <c r="E37" s="1">
         <f>SUM(E2:E36)</f>
-        <v>837300</v>
+        <v>833300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Delete budget item "Sadi basta"
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,8 +8,8 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H36</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1039,115 +1039,95 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>18d2728f</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B32" t="str">
-        <v>Sadi basta</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D32" s="1">
-        <v>25000</v>
+        <v>2000</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Baste k sadiya</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>d1aee56d</v>
+        <v>04ece648</v>
       </c>
       <c r="B33" t="str">
-        <v>Shireen Dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D33" s="1">
-        <v>2000</v>
+        <v>105000</v>
       </c>
       <c r="E33" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F33" t="str">
-        <v>Shireen Dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>04ece648</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B34" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C34" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>105000</v>
+        <v>6190</v>
       </c>
       <c r="E34" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F34" t="str">
-        <v>venue for reception</v>
+        <v>Prewedding dress</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>bd5f8d26</v>
+        <v>db4969e8</v>
       </c>
       <c r="B35" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="C35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D35" s="1">
-        <v>6190</v>
+        <v>5100</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>Prewedding dress</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>db4969e8</v>
-      </c>
-      <c r="B36" t="str">
         <v>Tushar Traders Oil</v>
       </c>
-      <c r="C36" t="str">
-        <v>Food &amp; Catering</v>
-      </c>
-      <c r="D36" s="1">
-        <v>5100</v>
-      </c>
-      <c r="E36" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F36" t="str">
-        <v>Tushar Traders Oil</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F36"/>
+  <autoFilter ref="A1:F35"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F35"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -1551,19 +1531,19 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>bd2ed5ab</v>
+        <v>762c8b3b</v>
       </c>
       <c r="B16" t="str">
-        <v>18d2728f</v>
+        <v>2c67b679</v>
       </c>
       <c r="C16" t="str">
-        <v>Sadi basta</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="D16" s="3">
         <v>46255</v>
       </c>
       <c r="E16" s="1">
-        <v>25000</v>
+        <v>24880</v>
       </c>
       <c r="F16" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -1572,50 +1552,50 @@
         <v>Debit Card</v>
       </c>
       <c r="H16" t="str">
-        <v>Paid baste sadi</v>
+        <v>Moolchand Sarees basta paid</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>762c8b3b</v>
+        <v>d478d6d7</v>
       </c>
       <c r="B17" t="str">
-        <v>2c67b679</v>
+        <v>1e95c55a</v>
       </c>
       <c r="C17" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="D17" s="3">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E17" s="1">
-        <v>24880</v>
+        <v>3675</v>
       </c>
       <c r="F17" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G17" t="str">
-        <v>Debit Card</v>
+        <v>UPI</v>
       </c>
       <c r="H17" t="str">
-        <v>Moolchand Sarees basta paid</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>d478d6d7</v>
+        <v>6d30e094</v>
       </c>
       <c r="B18" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="C18" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="D18" s="3">
         <v>46256</v>
       </c>
       <c r="E18" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="F18" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1629,45 +1609,45 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>6d30e094</v>
+        <v>04a382c3</v>
       </c>
       <c r="B19" t="str">
-        <v>aa710190</v>
+        <v>7896f0b1</v>
       </c>
       <c r="C19" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="D19" s="3">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E19" s="1">
-        <v>1500</v>
+        <v>24000</v>
       </c>
       <c r="F19" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G19" t="str">
-        <v>UPI</v>
+        <v>Debit Card</v>
       </c>
       <c r="H19" t="str">
-        <v>paid</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>04a382c3</v>
+        <v>b83ec348</v>
       </c>
       <c r="B20" t="str">
-        <v>7896f0b1</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="C20" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="D20" s="3">
         <v>46257</v>
       </c>
       <c r="E20" s="1">
-        <v>24000</v>
+        <v>12150</v>
       </c>
       <c r="F20" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -1676,128 +1656,128 @@
         <v>Debit Card</v>
       </c>
       <c r="H20" t="str">
-        <v>Paid</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>b83ec348</v>
+        <v>965c1bf2</v>
       </c>
       <c r="B21" t="str">
-        <v>d5fe8bfd</v>
+        <v>d1aee56d</v>
       </c>
       <c r="C21" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="D21" s="3">
         <v>46257</v>
       </c>
       <c r="E21" s="1">
-        <v>12150</v>
+        <v>2000</v>
       </c>
       <c r="F21" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G21" t="str">
-        <v>Debit Card</v>
+        <v>UPI</v>
       </c>
       <c r="H21" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Shireen Dress paid</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>965c1bf2</v>
+        <v>79903b8b</v>
       </c>
       <c r="B22" t="str">
-        <v>d1aee56d</v>
+        <v>7e3ae131</v>
       </c>
       <c r="C22" t="str">
-        <v>Shireen Dress</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
       <c r="D22" s="3">
         <v>46257</v>
       </c>
       <c r="E22" s="1">
-        <v>2000</v>
+        <v>4080</v>
       </c>
       <c r="F22" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G22" t="str">
         <v>UPI</v>
       </c>
       <c r="H22" t="str">
-        <v>Shireen Dress paid</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>79903b8b</v>
+        <v>109c6f27</v>
       </c>
       <c r="B23" t="str">
-        <v>7e3ae131</v>
+        <v>4e1fe7bf</v>
       </c>
       <c r="C23" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
+        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
       </c>
       <c r="D23" s="3">
         <v>46257</v>
       </c>
       <c r="E23" s="1">
-        <v>4080</v>
+        <v>1000</v>
       </c>
       <c r="F23" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G23" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H23" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
+        <v>advance</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>109c6f27</v>
+        <v>b5b081de</v>
       </c>
       <c r="B24" t="str">
-        <v>4e1fe7bf</v>
+        <v>1bb495b6</v>
       </c>
       <c r="C24" t="str">
-        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
+        <v>23 Aug Basta lunch at Shahidawat</v>
       </c>
       <c r="D24" s="3">
         <v>46257</v>
       </c>
       <c r="E24" s="1">
-        <v>1000</v>
+        <v>2545</v>
       </c>
       <c r="F24" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G24" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H24" t="str">
-        <v>advance</v>
+        <v>23 Aug Basta lunch paid</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>b5b081de</v>
+        <v>de8adadf</v>
       </c>
       <c r="B25" t="str">
-        <v>1bb495b6</v>
+        <v>a036f9f7</v>
       </c>
       <c r="C25" t="str">
-        <v>23 Aug Basta lunch at Shahidawat</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="D25" s="3">
         <v>46257</v>
       </c>
       <c r="E25" s="1">
-        <v>2545</v>
+        <v>550</v>
       </c>
       <c r="F25" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1806,128 +1786,128 @@
         <v>UPI</v>
       </c>
       <c r="H25" t="str">
-        <v>23 Aug Basta lunch paid</v>
+        <v>Bangal</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>de8adadf</v>
+        <v>c3d399da</v>
       </c>
       <c r="B26" t="str">
-        <v>a036f9f7</v>
+        <v>985ce939</v>
       </c>
       <c r="C26" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
       <c r="D26" s="3">
         <v>46257</v>
       </c>
       <c r="E26" s="1">
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="F26" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G26" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H26" t="str">
-        <v>Bangal</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>c3d399da</v>
+        <v>dccde075</v>
       </c>
       <c r="B27" t="str">
-        <v>985ce939</v>
+        <v>0e8bf89b</v>
       </c>
       <c r="C27" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="D27" s="3">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="E27" s="1">
-        <v>1300</v>
+        <v>2200</v>
       </c>
       <c r="F27" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G27" t="str">
         <v>Cash</v>
       </c>
       <c r="H27" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>dccde075</v>
+        <v>3c9c77ed</v>
       </c>
       <c r="B28" t="str">
-        <v>0e8bf89b</v>
+        <v>0421ab42</v>
       </c>
       <c r="C28" t="str">
-        <v>Bari ka saman</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="D28" s="3">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="E28" s="1">
-        <v>2200</v>
+        <v>4000</v>
       </c>
       <c r="F28" t="str">
         <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G28" t="str">
-        <v>Cash</v>
+        <v>Debit Card</v>
       </c>
       <c r="H28" t="str">
-        <v>paid</v>
+        <v>Petrol Paid</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>3c9c77ed</v>
+        <v>bbfbed2b</v>
       </c>
       <c r="B29" t="str">
-        <v>0421ab42</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="C29" t="str">
-        <v>Petrol Glanza</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="D29" s="3">
-        <v>46261</v>
+        <v>46263</v>
       </c>
       <c r="E29" s="1">
-        <v>4000</v>
+        <v>8649</v>
       </c>
       <c r="F29" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G29" t="str">
-        <v>Debit Card</v>
+        <v>UPI</v>
       </c>
       <c r="H29" t="str">
-        <v>Petrol Paid</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>bbfbed2b</v>
+        <v>c9cf6d4a</v>
       </c>
       <c r="B30" t="str">
-        <v>eebc3aaf</v>
+        <v>db4969e8</v>
       </c>
       <c r="C30" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="D30" s="3">
         <v>46263</v>
       </c>
       <c r="E30" s="1">
-        <v>8649</v>
+        <v>5100</v>
       </c>
       <c r="F30" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1941,19 +1921,19 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>c9cf6d4a</v>
+        <v>9c9ac50b</v>
       </c>
       <c r="B31" t="str">
-        <v>db4969e8</v>
+        <v>0beedebe</v>
       </c>
       <c r="C31" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="D31" s="3">
         <v>46263</v>
       </c>
       <c r="E31" s="1">
-        <v>5100</v>
+        <v>4600</v>
       </c>
       <c r="F31" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1962,24 +1942,24 @@
         <v>UPI</v>
       </c>
       <c r="H31" t="str">
-        <v>paid</v>
+        <v>Bhavesh Treaders (kirana) paid</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>9c9ac50b</v>
+        <v>cda2807c</v>
       </c>
       <c r="B32" t="str">
-        <v>0beedebe</v>
+        <v>e6b755dc</v>
       </c>
       <c r="C32" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="D32" s="3">
         <v>46263</v>
       </c>
       <c r="E32" s="1">
-        <v>4600</v>
+        <v>575</v>
       </c>
       <c r="F32" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1988,24 +1968,24 @@
         <v>UPI</v>
       </c>
       <c r="H32" t="str">
-        <v>Bhavesh Treaders (kirana) paid</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>cda2807c</v>
+        <v>62d1ce54</v>
       </c>
       <c r="B33" t="str">
-        <v>e6b755dc</v>
+        <v>89c1b231</v>
       </c>
       <c r="C33" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="D33" s="3">
         <v>46263</v>
       </c>
       <c r="E33" s="1">
-        <v>575</v>
+        <v>3345</v>
       </c>
       <c r="F33" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2014,76 +1994,76 @@
         <v>UPI</v>
       </c>
       <c r="H33" t="str">
-        <v>paid</v>
+        <v>Pravin Masal Paid</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>62d1ce54</v>
+        <v>13ce4f28</v>
       </c>
       <c r="B34" t="str">
-        <v>89c1b231</v>
+        <v>1aa31869</v>
       </c>
       <c r="C34" t="str">
-        <v>Pravin Masale</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="D34" s="3">
         <v>46263</v>
       </c>
       <c r="E34" s="1">
-        <v>3345</v>
+        <v>270</v>
       </c>
       <c r="F34" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G34" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H34" t="str">
-        <v>Pravin Masal Paid</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>13ce4f28</v>
+        <v>c2ac5cbf</v>
       </c>
       <c r="B35" t="str">
-        <v>1aa31869</v>
+        <v>05d27deb</v>
       </c>
       <c r="C35" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="D35" s="3">
         <v>46263</v>
       </c>
       <c r="E35" s="1">
-        <v>270</v>
+        <v>1124</v>
       </c>
       <c r="F35" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G35" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H35" t="str">
-        <v/>
+        <v>Cream House Lunch paid</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>c2ac5cbf</v>
+        <v>a7faa1c7</v>
       </c>
       <c r="B36" t="str">
-        <v>05d27deb</v>
+        <v>beb44857</v>
       </c>
       <c r="C36" t="str">
-        <v>Cream House Lunch</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="D36" s="3">
         <v>46263</v>
       </c>
       <c r="E36" s="1">
-        <v>1124</v>
+        <v>10000</v>
       </c>
       <c r="F36" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2092,46 +2072,20 @@
         <v>UPI</v>
       </c>
       <c r="H36" t="str">
-        <v>Cream House Lunch paid</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>a7faa1c7</v>
-      </c>
-      <c r="B37" t="str">
-        <v>beb44857</v>
-      </c>
-      <c r="C37" t="str">
-        <v>Pratap films and Photography</v>
-      </c>
-      <c r="D37" s="3">
-        <v>46263</v>
-      </c>
-      <c r="E37" s="1">
-        <v>10000</v>
-      </c>
-      <c r="F37" t="str">
-        <v>Asif Sayyed (Son)</v>
-      </c>
-      <c r="G37" t="str">
-        <v>UPI</v>
-      </c>
-      <c r="H37" t="str">
         <v>second installment</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H37"/>
+  <autoFilter ref="A1:H36"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H36"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E36"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2729,17 +2683,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Sadi basta</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B32" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C32" s="1">
-        <v>25000</v>
+        <v>2000</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>25000</v>
+        <v>2000</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -2748,55 +2702,55 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Shireen Dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C33" s="1">
-        <v>2000</v>
+        <v>105000</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>15000</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B34" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>105000</v>
+        <v>6190</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>6190</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Tushar Traders Oil</v>
       </c>
       <c r="B35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C35" s="1">
-        <v>6190</v>
+        <v>5100</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>5100</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -2805,43 +2759,24 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Tushar Traders Oil</v>
-      </c>
-      <c r="B36" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Total</v>
       </c>
       <c r="C36" s="1">
-        <v>5100</v>
+        <f>SUM(C2:C35)</f>
+        <v>1102866</v>
       </c>
       <c r="D36" s="1">
-        <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <f>SUM(D2:D35)</f>
+        <v>269566</v>
       </c>
       <c r="E36" s="1">
-        <f>C36-D36</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>Total</v>
-      </c>
-      <c r="C37" s="1">
-        <f>SUM(C2:C36)</f>
-        <v>1127866</v>
-      </c>
-      <c r="D37" s="1">
-        <f>SUM(D2:D36)</f>
-        <v>294566</v>
-      </c>
-      <c r="E37" s="1">
-        <f>SUM(E2:E36)</f>
+        <f>SUM(E2:E35)</f>
         <v>833300</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update payment: ₹1,500.00 by Asif Sayyed (Son) for Invitation Card (Shubham)
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -1583,45 +1583,45 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>6d30e094</v>
+        <v>04a382c3</v>
       </c>
       <c r="B18" t="str">
-        <v>aa710190</v>
+        <v>7896f0b1</v>
       </c>
       <c r="C18" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="D18" s="3">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E18" s="1">
-        <v>1500</v>
+        <v>24000</v>
       </c>
       <c r="F18" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G18" t="str">
-        <v>UPI</v>
+        <v>Debit Card</v>
       </c>
       <c r="H18" t="str">
-        <v>paid</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>04a382c3</v>
+        <v>b83ec348</v>
       </c>
       <c r="B19" t="str">
-        <v>7896f0b1</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="C19" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="D19" s="3">
         <v>46257</v>
       </c>
       <c r="E19" s="1">
-        <v>24000</v>
+        <v>12150</v>
       </c>
       <c r="F19" t="str">
         <v>Umar Sayyed (Father)</v>
@@ -1630,128 +1630,128 @@
         <v>Debit Card</v>
       </c>
       <c r="H19" t="str">
-        <v>Paid</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>b83ec348</v>
+        <v>965c1bf2</v>
       </c>
       <c r="B20" t="str">
-        <v>d5fe8bfd</v>
+        <v>d1aee56d</v>
       </c>
       <c r="C20" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="D20" s="3">
         <v>46257</v>
       </c>
       <c r="E20" s="1">
-        <v>12150</v>
+        <v>2000</v>
       </c>
       <c r="F20" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G20" t="str">
-        <v>Debit Card</v>
+        <v>UPI</v>
       </c>
       <c r="H20" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Shireen Dress paid</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>965c1bf2</v>
+        <v>79903b8b</v>
       </c>
       <c r="B21" t="str">
-        <v>d1aee56d</v>
+        <v>7e3ae131</v>
       </c>
       <c r="C21" t="str">
-        <v>Shireen Dress</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
       </c>
       <c r="D21" s="3">
         <v>46257</v>
       </c>
       <c r="E21" s="1">
-        <v>2000</v>
+        <v>4080</v>
       </c>
       <c r="F21" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G21" t="str">
         <v>UPI</v>
       </c>
       <c r="H21" t="str">
-        <v>Shireen Dress paid</v>
+        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>79903b8b</v>
+        <v>109c6f27</v>
       </c>
       <c r="B22" t="str">
-        <v>7e3ae131</v>
+        <v>4e1fe7bf</v>
       </c>
       <c r="C22" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress</v>
+        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
       </c>
       <c r="D22" s="3">
         <v>46257</v>
       </c>
       <c r="E22" s="1">
-        <v>4080</v>
+        <v>1000</v>
       </c>
       <c r="F22" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G22" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H22" t="str">
-        <v>(Mumbai Textile &amp; Parag) Bade Abba, Anis, Navshad &amp; Salima Dress paid</v>
+        <v>advance</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>109c6f27</v>
+        <v>b5b081de</v>
       </c>
       <c r="B23" t="str">
-        <v>4e1fe7bf</v>
+        <v>1bb495b6</v>
       </c>
       <c r="C23" t="str">
-        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
+        <v>23 Aug Basta lunch at Shahidawat</v>
       </c>
       <c r="D23" s="3">
         <v>46257</v>
       </c>
       <c r="E23" s="1">
-        <v>1000</v>
+        <v>2545</v>
       </c>
       <c r="F23" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G23" t="str">
-        <v>Cash</v>
+        <v>UPI</v>
       </c>
       <c r="H23" t="str">
-        <v>advance</v>
+        <v>23 Aug Basta lunch paid</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>b5b081de</v>
+        <v>de8adadf</v>
       </c>
       <c r="B24" t="str">
-        <v>1bb495b6</v>
+        <v>a036f9f7</v>
       </c>
       <c r="C24" t="str">
-        <v>23 Aug Basta lunch at Shahidawat</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="D24" s="3">
         <v>46257</v>
       </c>
       <c r="E24" s="1">
-        <v>2545</v>
+        <v>550</v>
       </c>
       <c r="F24" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -1760,111 +1760,111 @@
         <v>UPI</v>
       </c>
       <c r="H24" t="str">
-        <v>23 Aug Basta lunch paid</v>
+        <v>Bangal</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>de8adadf</v>
+        <v>c3d399da</v>
       </c>
       <c r="B25" t="str">
-        <v>a036f9f7</v>
+        <v>985ce939</v>
       </c>
       <c r="C25" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
       <c r="D25" s="3">
         <v>46257</v>
       </c>
       <c r="E25" s="1">
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="F25" t="str">
-        <v>Asif Sayyed (Son)</v>
+        <v>Waheeda (mother)</v>
       </c>
       <c r="G25" t="str">
-        <v>UPI</v>
+        <v>Cash</v>
       </c>
       <c r="H25" t="str">
-        <v>Bangal</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>c3d399da</v>
+        <v>dccde075</v>
       </c>
       <c r="B26" t="str">
-        <v>985ce939</v>
+        <v>0e8bf89b</v>
       </c>
       <c r="C26" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="D26" s="3">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="E26" s="1">
-        <v>1300</v>
+        <v>2200</v>
       </c>
       <c r="F26" t="str">
-        <v>Waheeda (mother)</v>
+        <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G26" t="str">
         <v>Cash</v>
       </c>
       <c r="H26" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>dccde075</v>
+        <v>3c9c77ed</v>
       </c>
       <c r="B27" t="str">
-        <v>0e8bf89b</v>
+        <v>0421ab42</v>
       </c>
       <c r="C27" t="str">
-        <v>Bari ka saman</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="D27" s="3">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="E27" s="1">
-        <v>2200</v>
+        <v>4000</v>
       </c>
       <c r="F27" t="str">
         <v>Umar Sayyed (Father)</v>
       </c>
       <c r="G27" t="str">
-        <v>Cash</v>
+        <v>Debit Card</v>
       </c>
       <c r="H27" t="str">
-        <v>paid</v>
+        <v>Petrol Paid</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>3c9c77ed</v>
+        <v>6d30e094</v>
       </c>
       <c r="B28" t="str">
-        <v>0421ab42</v>
+        <v>aa710190</v>
       </c>
       <c r="C28" t="str">
-        <v>Petrol Glanza</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="D28" s="3">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="E28" s="1">
-        <v>4000</v>
+        <v>1500</v>
       </c>
       <c r="F28" t="str">
-        <v>Umar Sayyed (Father)</v>
+        <v>Asif Sayyed (Son)</v>
       </c>
       <c r="G28" t="str">
-        <v>Debit Card</v>
+        <v>UPI</v>
       </c>
       <c r="H28" t="str">
-        <v>Petrol Paid</v>
+        <v>paid</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Record payment: ₹10,300.00 by Umar Sayyed (Father) for (Famous & Libas Tailor)Silaee for Abba, Didi, Asif & irfan Bhaijan
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H37</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1127,7 +1127,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2075,10 +2075,36 @@
         <v>second installment</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>6297fd78</v>
+      </c>
+      <c r="B37" t="str">
+        <v>4e1fe7bf</v>
+      </c>
+      <c r="C37" t="str">
+        <v>(Famous &amp; Libas Tailor)Silaee for Abba, Didi, Asif &amp; irfan Bhaijan</v>
+      </c>
+      <c r="D37" s="3">
+        <v>46266</v>
+      </c>
+      <c r="E37" s="1">
+        <v>10300</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G37" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H37" t="str">
+        <v>full payment done</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H36"/>
+  <autoFilter ref="A1:H37"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2123,11 +2149,11 @@
       </c>
       <c r="D2" s="1">
         <f>SUMIF('Payments'!$C:$C,$A2,'Payments'!$E:$E)</f>
-        <v>1000</v>
+        <v>11300</v>
       </c>
       <c r="E2" s="1">
         <f>C2-D2</f>
-        <v>10300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -2767,11 +2793,11 @@
       </c>
       <c r="D36" s="1">
         <f>SUM(D2:D35)</f>
-        <v>269566</v>
+        <v>279866</v>
       </c>
       <c r="E36" s="1">
         <f>SUM(E2:E35)</f>
-        <v>833300</v>
+        <v>823000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Aluminum Shop Partition — ₹23,000.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H37</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -519,608 +519,628 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>985ce939</v>
+        <v>aaedf833</v>
       </c>
       <c r="B6" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Aluminum Shop Partition</v>
       </c>
       <c r="C6" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D6" s="1">
-        <v>1300</v>
+        <v>23000</v>
       </c>
       <c r="E6" s="2" t="str">
-        <v/>
+        <v>8446627171</v>
       </c>
       <c r="F6" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Aluminum Shop Partition</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>a036f9f7</v>
+        <v>985ce939</v>
       </c>
       <c r="B7" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
       <c r="C7" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D7" s="1">
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="E7" s="2" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>0e8bf89b</v>
+        <v>a036f9f7</v>
       </c>
       <c r="B8" t="str">
-        <v>Bari ka saman</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="C8" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D8" s="1">
-        <v>2200</v>
+        <v>550</v>
       </c>
       <c r="E8" s="2" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v>Bari ka saman</v>
+        <v>Arbiya Bangals</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>1aa31869</v>
+        <v>0e8bf89b</v>
       </c>
       <c r="B9" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="C9" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="D9" s="1">
-        <v>270</v>
+        <v>2200</v>
       </c>
       <c r="E9" s="2" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Bari ka saman</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>0beedebe</v>
+        <v>1aa31869</v>
       </c>
       <c r="B10" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="C10" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D10" s="1">
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="E10" s="2" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>05d27deb</v>
+        <v>0beedebe</v>
       </c>
       <c r="B11" t="str">
-        <v>Cream House Lunch</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="C11" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D11" s="1">
-        <v>1124</v>
+        <v>4600</v>
       </c>
       <c r="E11" s="2" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>Cream House Lunch</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>631875ca</v>
+        <v>05d27deb</v>
       </c>
       <c r="B12" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="C12" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D12" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F12" t="str">
-        <v>Hall decoration</v>
+        <v>Cream House Lunch</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B13" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C13" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D13" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E13" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F13" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B14" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D14" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F14" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B15" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C15" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D15" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F15" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B16" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C16" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D16" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E16" s="2" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B17" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C17" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D17" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E17" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F17" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>aa710190</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B18" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C18" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D18" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v>7385125161</v>
+        <v>9226111899</v>
       </c>
       <c r="F18" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B19" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C19" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D19" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F19" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B20" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C20" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D20" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F20" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B21" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D21" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E21" s="2" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B22" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D22" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E22" s="2" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B23" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D23" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>eebc3aaf</v>
+        <v>a78dd739</v>
       </c>
       <c r="B24" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C24" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D24" s="1">
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B25" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C25" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D25" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B26" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C26" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D26" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B27" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D27" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B28" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C28" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D28" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>beb44857</v>
+        <v>0421ab42</v>
       </c>
       <c r="B29" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C29" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D29" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E29" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F29" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B30" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C30" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D30" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E30" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F30" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B31" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C31" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D31" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E31" s="2" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B32" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D32" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B33" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C33" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D33" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E33" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F33" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B34" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D34" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E34" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F34" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B35" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C35" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E35" s="2" t="str">
         <v/>
       </c>
       <c r="F35" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B36" t="str">
         <v>Tushar Traders Oil</v>
       </c>
+      <c r="C36" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D36" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E36" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F35"/>
+  <autoFilter ref="A1:F36"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2111,7 +2131,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2215,36 +2235,36 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Arbiya &amp; Didi Sangle</v>
+        <v>Aluminum Shop Partition</v>
       </c>
       <c r="B6" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C6" s="1">
-        <v>1300</v>
+        <v>23000</v>
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>0</v>
+        <v>23000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Arbiya Bangals</v>
+        <v>Arbiya &amp; Didi Sangle</v>
       </c>
       <c r="B7" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C7" s="1">
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="D7" s="1">
         <f>SUMIF('Payments'!$C:$C,$A7,'Payments'!$E:$E)</f>
-        <v>550</v>
+        <v>1300</v>
       </c>
       <c r="E7" s="1">
         <f>C7-D7</f>
@@ -2253,17 +2273,17 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Bari ka saman</v>
+        <v>Arbiya Bangals</v>
       </c>
       <c r="B8" t="str">
-        <v>Gifts &amp; Return Gifts</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C8" s="1">
-        <v>2200</v>
+        <v>550</v>
       </c>
       <c r="D8" s="1">
         <f>SUMIF('Payments'!$C:$C,$A8,'Payments'!$E:$E)</f>
-        <v>2200</v>
+        <v>550</v>
       </c>
       <c r="E8" s="1">
         <f>C8-D8</f>
@@ -2272,17 +2292,17 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Bhavesh Treaders (karele &amp; javas)</v>
+        <v>Bari ka saman</v>
       </c>
       <c r="B9" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Gifts &amp; Return Gifts</v>
       </c>
       <c r="C9" s="1">
-        <v>270</v>
+        <v>2200</v>
       </c>
       <c r="D9" s="1">
         <f>SUMIF('Payments'!$C:$C,$A9,'Payments'!$E:$E)</f>
-        <v>270</v>
+        <v>2200</v>
       </c>
       <c r="E9" s="1">
         <f>C9-D9</f>
@@ -2291,17 +2311,17 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Bhavesh Treaders (kirana)</v>
+        <v>Bhavesh Treaders (karele &amp; javas)</v>
       </c>
       <c r="B10" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C10" s="1">
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="D10" s="1">
         <f>SUMIF('Payments'!$C:$C,$A10,'Payments'!$E:$E)</f>
-        <v>4600</v>
+        <v>270</v>
       </c>
       <c r="E10" s="1">
         <f>C10-D10</f>
@@ -2310,17 +2330,17 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Cream House Lunch</v>
+        <v>Bhavesh Treaders (kirana)</v>
       </c>
       <c r="B11" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C11" s="1">
-        <v>1124</v>
+        <v>4600</v>
       </c>
       <c r="D11" s="1">
         <f>SUMIF('Payments'!$C:$C,$A11,'Payments'!$E:$E)</f>
-        <v>1124</v>
+        <v>4600</v>
       </c>
       <c r="E11" s="1">
         <f>C11-D11</f>
@@ -2329,55 +2349,55 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="B12" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C12" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>1124</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>128000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B13" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C13" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B14" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C14" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
@@ -2386,17 +2406,17 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B15" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C15" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -2405,17 +2425,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B16" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C16" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -2424,55 +2444,55 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B17" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C17" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B18" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C18" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>50000</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B19" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C19" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
@@ -2481,17 +2501,17 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B20" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C20" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -2500,17 +2520,17 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B21" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C21" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -2519,17 +2539,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C22" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2538,17 +2558,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C23" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2557,17 +2577,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B24" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C24" s="1">
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>400</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2576,17 +2596,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B25" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C25" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -2595,17 +2615,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B26" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C26" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -2614,17 +2634,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B27" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C27" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -2633,17 +2653,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B28" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C28" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -2652,55 +2672,55 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B29" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C29" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>20000</v>
+        <v>4000</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
-        <v>80000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B30" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C30" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>20000</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
-        <v>0</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B31" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C31" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
@@ -2709,17 +2729,17 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B32" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C32" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -2728,55 +2748,55 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B33" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C33" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C34" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B35" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
@@ -2785,24 +2805,43 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C36" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D36" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E36" s="1">
+        <f>C36-D36</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
         <v>Total</v>
       </c>
-      <c r="C36" s="1">
-        <f>SUM(C2:C35)</f>
-        <v>1102866</v>
-      </c>
-      <c r="D36" s="1">
-        <f>SUM(D2:D35)</f>
+      <c r="C37" s="1">
+        <f>SUM(C2:C36)</f>
+        <v>1125866</v>
+      </c>
+      <c r="D37" s="1">
+        <f>SUM(D2:D36)</f>
         <v>279866</v>
       </c>
-      <c r="E36" s="1">
-        <f>SUM(E2:E35)</f>
-        <v>823000</v>
+      <c r="E37" s="1">
+        <f>SUM(E2:E36)</f>
+        <v>846000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹15,000.00 by Asif Sayyed (Son) for Aluminum Shop Partition
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H38</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1147,7 +1147,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2121,10 +2121,36 @@
         <v>full payment done</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>0bd24ffb</v>
+      </c>
+      <c r="B38" t="str">
+        <v>aaedf833</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Aluminum Shop Partition</v>
+      </c>
+      <c r="D38" s="3">
+        <v>46271</v>
+      </c>
+      <c r="E38" s="1">
+        <v>15000</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G38" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Paid Advance</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H37"/>
+  <autoFilter ref="A1:H38"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2245,11 +2271,11 @@
       </c>
       <c r="D6" s="1">
         <f>SUMIF('Payments'!$C:$C,$A6,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="E6" s="1">
         <f>C6-D6</f>
-        <v>23000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="7">
@@ -2832,11 +2858,11 @@
       </c>
       <c r="D37" s="1">
         <f>SUM(D2:D36)</f>
-        <v>279866</v>
+        <v>294866</v>
       </c>
       <c r="E37" s="1">
         <f>SUM(E2:E36)</f>
-        <v>846000</v>
+        <v>831000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Mummy sadi — ₹1,600.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H38</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -899,248 +899,268 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B25" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C25" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B26" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C26" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D26" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B27" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C27" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D27" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B28" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D28" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B29" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C29" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D29" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>beb44857</v>
+        <v>0421ab42</v>
       </c>
       <c r="B30" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C30" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D30" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E30" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F30" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B31" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C31" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D31" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E31" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F31" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B32" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C32" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D32" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E32" s="2" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B33" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D33" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B34" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C34" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D34" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E34" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F34" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B35" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D35" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E35" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F35" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>db4969e8</v>
+        <v>bd5f8d26</v>
       </c>
       <c r="B36" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="C36" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D36" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E36" s="2" t="str">
         <v/>
       </c>
       <c r="F36" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>db4969e8</v>
+      </c>
+      <c r="B37" t="str">
         <v>Tushar Traders Oil</v>
       </c>
+      <c r="C37" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="D37" s="1">
+        <v>5100</v>
+      </c>
+      <c r="E37" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F36"/>
+  <autoFilter ref="A1:F37"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2157,7 +2177,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2622,36 +2642,36 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B25" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>0</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B26" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C26" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -2660,17 +2680,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B27" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C27" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -2679,17 +2699,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B28" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C28" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -2698,17 +2718,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B29" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C29" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -2717,55 +2737,55 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B30" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C30" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>20000</v>
+        <v>4000</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
-        <v>80000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B31" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C31" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>20000</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
-        <v>0</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B32" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C32" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
@@ -2774,17 +2794,17 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B33" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C33" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -2793,55 +2813,55 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B34" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C34" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B35" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C35" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B36" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C36" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
@@ -2850,24 +2870,43 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C37" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D37" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E37" s="1">
+        <f>C37-D37</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
         <v>Total</v>
       </c>
-      <c r="C37" s="1">
-        <f>SUM(C2:C36)</f>
-        <v>1125866</v>
-      </c>
-      <c r="D37" s="1">
-        <f>SUM(D2:D36)</f>
+      <c r="C38" s="1">
+        <f>SUM(C2:C37)</f>
+        <v>1127466</v>
+      </c>
+      <c r="D38" s="1">
+        <f>SUM(D2:D37)</f>
         <v>294866</v>
       </c>
-      <c r="E37" s="1">
-        <f>SUM(E2:E36)</f>
-        <v>831000</v>
+      <c r="E38" s="1">
+        <f>SUM(E2:E37)</f>
+        <v>832600</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹1,600.00 by Umar Sayyed (Father) for Mummy sadi
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H39</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1167,7 +1167,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2167,10 +2167,36 @@
         <v>Paid Advance</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>a1d6ea2f</v>
+      </c>
+      <c r="B39" t="str">
+        <v>30b69ec5</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Mummy sadi</v>
+      </c>
+      <c r="D39" s="3">
+        <v>46272</v>
+      </c>
+      <c r="E39" s="1">
+        <v>1600</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Umar Sayyed (Father)</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Cash</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H38"/>
+  <autoFilter ref="A1:H39"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H39"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2652,11 +2678,11 @@
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
-        <v>1600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -2897,11 +2923,11 @@
       </c>
       <c r="D38" s="1">
         <f>SUM(D2:D37)</f>
-        <v>294866</v>
+        <v>296466</v>
       </c>
       <c r="E38" s="1">
         <f>SUM(E2:E37)</f>
-        <v>832600</v>
+        <v>831000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add budget item: Colour & plumber — ₹800.00
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -8,7 +8,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H39</definedName>
   </definedNames>
 </workbook>
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -639,528 +639,548 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>05d27deb</v>
+        <v>2a74d868</v>
       </c>
       <c r="B12" t="str">
-        <v>Cream House Lunch</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="C12" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D12" s="1">
-        <v>1124</v>
+        <v>800</v>
       </c>
       <c r="E12" s="2" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>Cream House Lunch</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>631875ca</v>
+        <v>05d27deb</v>
       </c>
       <c r="B13" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="C13" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D13" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="E13" s="2" t="str">
-        <v>9536673041</v>
+        <v/>
       </c>
       <c r="F13" t="str">
-        <v>Hall decoration</v>
+        <v>Cream House Lunch</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>d5fe8bfd</v>
+        <v>631875ca</v>
       </c>
       <c r="B14" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="C14" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="D14" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v/>
+        <v>9536673041</v>
       </c>
       <c r="F14" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Hall decoration</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>9a8449e7</v>
+        <v>d5fe8bfd</v>
       </c>
       <c r="B15" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="C15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D15" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v>9665012980</v>
+        <v/>
       </c>
       <c r="F15" t="str">
-        <v>Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>070f7b33</v>
+        <v>9a8449e7</v>
       </c>
       <c r="B16" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="C16" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D16" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E16" s="2" t="str">
-        <v/>
+        <v>9665012980</v>
       </c>
       <c r="F16" t="str">
-        <v>Blue Nile &amp; Seasons mall</v>
+        <v>Groom Reception dress</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>209d43b7</v>
+        <v>070f7b33</v>
       </c>
       <c r="B17" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="C17" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D17" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E17" s="2" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Blue Nile &amp; Seasons mall</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>168b7bbd</v>
+        <v>209d43b7</v>
       </c>
       <c r="B18" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="C18" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="D18" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="E18" s="2" t="str">
-        <v>9226111899</v>
+        <v/>
       </c>
       <c r="F18" t="str">
-        <v>Reception food</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>aa710190</v>
+        <v>168b7bbd</v>
       </c>
       <c r="B19" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="C19" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D19" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v>7385125161</v>
+        <v>9226111899</v>
       </c>
       <c r="F19" t="str">
-        <v>Invitation Card (Shubham)  100</v>
+        <v>Reception food</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>1e95c55a</v>
+        <v>aa710190</v>
       </c>
       <c r="B20" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="C20" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="D20" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E20" s="2" t="str">
-        <v>9890326266</v>
+        <v>7385125161</v>
       </c>
       <c r="F20" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)  100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>c7e8b352</v>
+        <v>1e95c55a</v>
       </c>
       <c r="B21" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="C21" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="D21" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E21" s="2" t="str">
-        <v/>
+        <v>9890326266</v>
       </c>
       <c r="F21" t="str">
-        <v>Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2c67b679</v>
+        <v>c7e8b352</v>
       </c>
       <c r="B22" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="C22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D22" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E22" s="2" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>Moolchand Sarees for basta</v>
+        <v>Bride reception dress</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>068998a3</v>
+        <v>2c67b679</v>
       </c>
       <c r="B23" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="C23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D23" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E23" s="2" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>Groom wedding dress</v>
+        <v>Moolchand Sarees for basta</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>a78dd739</v>
+        <v>068998a3</v>
       </c>
       <c r="B24" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="C24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D24" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E24" s="2" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>Shoes</v>
+        <v>Groom wedding dress</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>30b69ec5</v>
+        <v>a78dd739</v>
       </c>
       <c r="B25" t="str">
-        <v>Mummy sadi</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="C25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D25" s="1">
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="E25" s="2" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>Shoes</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>eebc3aaf</v>
+        <v>30b69ec5</v>
       </c>
       <c r="B26" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="C26" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D26" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E26" s="2" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>e6b755dc</v>
+        <v>eebc3aaf</v>
       </c>
       <c r="B27" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="C27" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="D27" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E27" s="2" t="str">
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>113a1c1a</v>
+        <v>e6b755dc</v>
       </c>
       <c r="B28" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="C28" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D28" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E28" s="2" t="str">
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>7896f0b1</v>
+        <v>113a1c1a</v>
       </c>
       <c r="B29" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="C29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D29" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E29" s="2" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>bride 3 dress</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>0421ab42</v>
+        <v>7896f0b1</v>
       </c>
       <c r="B30" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="C30" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D30" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E30" s="2" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>beb44857</v>
+        <v>0421ab42</v>
       </c>
       <c r="B31" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="C31" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D31" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="E31" s="2" t="str">
-        <v>9021598286</v>
+        <v/>
       </c>
       <c r="F31" t="str">
-        <v>Photography cost</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>89c1b231</v>
+        <v>beb44857</v>
       </c>
       <c r="B32" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="C32" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="D32" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="E32" s="2" t="str">
-        <v/>
+        <v>9021598286</v>
       </c>
       <c r="F32" t="str">
-        <v>Pravin Masale</v>
+        <v>Photography cost</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>6d180155</v>
+        <v>89c1b231</v>
       </c>
       <c r="B33" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="C33" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="D33" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E33" s="2" t="str">
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>d1aee56d</v>
+        <v>6d180155</v>
       </c>
       <c r="B34" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="C34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="D34" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E34" s="2" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>04ece648</v>
+        <v>d1aee56d</v>
       </c>
       <c r="B35" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="C35" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="D35" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="E35" s="2" t="str">
-        <v>9850444117</v>
+        <v/>
       </c>
       <c r="F35" t="str">
-        <v>venue for reception</v>
+        <v>Shireen Dress</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>bd5f8d26</v>
+        <v>04ece648</v>
       </c>
       <c r="B36" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="C36" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="D36" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="E36" s="2" t="str">
-        <v/>
+        <v>9850444117</v>
       </c>
       <c r="F36" t="str">
-        <v>Prewedding dress</v>
+        <v>venue for reception</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
+        <v>bd5f8d26</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Star Bazaar - Prewedding dress</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Clothing &amp; Jewellery</v>
+      </c>
+      <c r="D37" s="1">
+        <v>6190</v>
+      </c>
+      <c r="E37" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v>Prewedding dress</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
         <v>db4969e8</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B38" t="str">
         <v>Tushar Traders Oil</v>
       </c>
-      <c r="C37" t="str">
+      <c r="C38" t="str">
         <v>Food &amp; Catering</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D38" s="1">
         <v>5100</v>
       </c>
-      <c r="E37" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F37" t="str">
+      <c r="E38" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
         <v>Tushar Traders Oil</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F37"/>
+  <autoFilter ref="A1:F38"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F38"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2203,7 +2223,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -2421,74 +2441,74 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Cream House Lunch</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="B12" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C12" s="1">
-        <v>1124</v>
+        <v>800</v>
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>1124</v>
+        <v>0</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>0</v>
+        <v>800</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Day night Flower Decoration - (hall)</v>
+        <v>Cream House Lunch</v>
       </c>
       <c r="B13" t="str">
-        <v>Decoration</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C13" s="1">
-        <v>143000</v>
+        <v>1124</v>
       </c>
       <c r="D13" s="1">
         <f>SUMIF('Payments'!$C:$C,$A13,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>1124</v>
       </c>
       <c r="E13" s="1">
         <f>C13-D13</f>
-        <v>128000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Famous cotton- Pathani 9</v>
+        <v>Day night Flower Decoration - (hall)</v>
       </c>
       <c r="B14" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Decoration</v>
       </c>
       <c r="C14" s="1">
-        <v>12150</v>
+        <v>143000</v>
       </c>
       <c r="D14" s="1">
         <f>SUMIF('Payments'!$C:$C,$A14,'Payments'!$E:$E)</f>
-        <v>12150</v>
+        <v>15000</v>
       </c>
       <c r="E14" s="1">
         <f>C14-D14</f>
-        <v>0</v>
+        <v>128000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Famous Tailor - Groom Reception dress</v>
+        <v>Famous cotton- Pathani 9</v>
       </c>
       <c r="B15" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C15" s="1">
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="D15" s="1">
         <f>SUMIF('Payments'!$C:$C,$A15,'Payments'!$E:$E)</f>
-        <v>10000</v>
+        <v>12150</v>
       </c>
       <c r="E15" s="1">
         <f>C15-D15</f>
@@ -2497,17 +2517,17 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Food at shopping time</v>
+        <v>Famous Tailor - Groom Reception dress</v>
       </c>
       <c r="B16" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C16" s="1">
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="D16" s="1">
         <f>SUMIF('Payments'!$C:$C,$A16,'Payments'!$E:$E)</f>
-        <v>2609</v>
+        <v>10000</v>
       </c>
       <c r="E16" s="1">
         <f>C16-D16</f>
@@ -2516,17 +2536,17 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Groom haircut and other saloon expences</v>
+        <v>Food at shopping time</v>
       </c>
       <c r="B17" t="str">
-        <v>Beauty &amp; Mehendi</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C17" s="1">
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="D17" s="1">
         <f>SUMIF('Payments'!$C:$C,$A17,'Payments'!$E:$E)</f>
-        <v>500</v>
+        <v>2609</v>
       </c>
       <c r="E17" s="1">
         <f>C17-D17</f>
@@ -2535,55 +2555,55 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Huseni Caterers</v>
+        <v>Groom haircut and other saloon expences</v>
       </c>
       <c r="B18" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Beauty &amp; Mehendi</v>
       </c>
       <c r="C18" s="1">
-        <v>575000</v>
+        <v>500</v>
       </c>
       <c r="D18" s="1">
         <f>SUMIF('Payments'!$C:$C,$A18,'Payments'!$E:$E)</f>
-        <v>50000</v>
+        <v>500</v>
       </c>
       <c r="E18" s="1">
         <f>C18-D18</f>
-        <v>525000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Invitation Card (Shubham)</v>
+        <v>Huseni Caterers</v>
       </c>
       <c r="B19" t="str">
-        <v>Invitations &amp; Printing</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C19" s="1">
-        <v>1500</v>
+        <v>575000</v>
       </c>
       <c r="D19" s="1">
         <f>SUMIF('Payments'!$C:$C,$A19,'Payments'!$E:$E)</f>
-        <v>1500</v>
+        <v>50000</v>
       </c>
       <c r="E19" s="1">
         <f>C19-D19</f>
-        <v>0</v>
+        <v>525000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Invitation Card (treaditional)</v>
+        <v>Invitation Card (Shubham)</v>
       </c>
       <c r="B20" t="str">
         <v>Invitations &amp; Printing</v>
       </c>
       <c r="C20" s="1">
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="D20" s="1">
         <f>SUMIF('Payments'!$C:$C,$A20,'Payments'!$E:$E)</f>
-        <v>3675</v>
+        <v>1500</v>
       </c>
       <c r="E20" s="1">
         <f>C20-D20</f>
@@ -2592,17 +2612,17 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Moolchand - Bride reception dress</v>
+        <v>Invitation Card (treaditional)</v>
       </c>
       <c r="B21" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Invitations &amp; Printing</v>
       </c>
       <c r="C21" s="1">
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="D21" s="1">
         <f>SUMIF('Payments'!$C:$C,$A21,'Payments'!$E:$E)</f>
-        <v>7604</v>
+        <v>3675</v>
       </c>
       <c r="E21" s="1">
         <f>C21-D21</f>
@@ -2611,17 +2631,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Moolchand Sarees basta</v>
+        <v>Moolchand - Bride reception dress</v>
       </c>
       <c r="B22" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C22" s="1">
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="D22" s="1">
         <f>SUMIF('Payments'!$C:$C,$A22,'Payments'!$E:$E)</f>
-        <v>24880</v>
+        <v>7604</v>
       </c>
       <c r="E22" s="1">
         <f>C22-D22</f>
@@ -2630,17 +2650,17 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Morya Collections - Groom wedding dress</v>
+        <v>Moolchand Sarees basta</v>
       </c>
       <c r="B23" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C23" s="1">
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="D23" s="1">
         <f>SUMIF('Payments'!$C:$C,$A23,'Payments'!$E:$E)</f>
-        <v>13680</v>
+        <v>24880</v>
       </c>
       <c r="E23" s="1">
         <f>C23-D23</f>
@@ -2649,17 +2669,17 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Morya mojadii</v>
+        <v>Morya Collections - Groom wedding dress</v>
       </c>
       <c r="B24" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C24" s="1">
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="D24" s="1">
         <f>SUMIF('Payments'!$C:$C,$A24,'Payments'!$E:$E)</f>
-        <v>400</v>
+        <v>13680</v>
       </c>
       <c r="E24" s="1">
         <f>C24-D24</f>
@@ -2668,17 +2688,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Mummy sadi</v>
+        <v>Morya mojadii</v>
       </c>
       <c r="B25" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C25" s="1">
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="D25" s="1">
         <f>SUMIF('Payments'!$C:$C,$A25,'Payments'!$E:$E)</f>
-        <v>1600</v>
+        <v>400</v>
       </c>
       <c r="E25" s="1">
         <f>C25-D25</f>
@@ -2687,17 +2707,17 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Navkar Sales Corporation</v>
+        <v>Mummy sadi</v>
       </c>
       <c r="B26" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C26" s="1">
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="D26" s="1">
         <f>SUMIF('Payments'!$C:$C,$A26,'Payments'!$E:$E)</f>
-        <v>8649</v>
+        <v>1600</v>
       </c>
       <c r="E26" s="1">
         <f>C26-D26</f>
@@ -2706,17 +2726,17 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>New Balaji Treaders</v>
+        <v>Navkar Sales Corporation</v>
       </c>
       <c r="B27" t="str">
         <v>Food &amp; Catering</v>
       </c>
       <c r="C27" s="1">
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="D27" s="1">
         <f>SUMIF('Payments'!$C:$C,$A27,'Payments'!$E:$E)</f>
-        <v>575</v>
+        <v>8649</v>
       </c>
       <c r="E27" s="1">
         <f>C27-D27</f>
@@ -2725,17 +2745,17 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Parag bride 3 dress</v>
+        <v>New Balaji Treaders</v>
       </c>
       <c r="B28" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C28" s="1">
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="D28" s="1">
         <f>SUMIF('Payments'!$C:$C,$A28,'Payments'!$E:$E)</f>
-        <v>5700</v>
+        <v>575</v>
       </c>
       <c r="E28" s="1">
         <f>C28-D28</f>
@@ -2744,17 +2764,17 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Parag Relative 20 dressed &amp; other cloths</v>
+        <v>Parag bride 3 dress</v>
       </c>
       <c r="B29" t="str">
         <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C29" s="1">
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="D29" s="1">
         <f>SUMIF('Payments'!$C:$C,$A29,'Payments'!$E:$E)</f>
-        <v>24000</v>
+        <v>5700</v>
       </c>
       <c r="E29" s="1">
         <f>C29-D29</f>
@@ -2763,17 +2783,17 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Petrol Glanza</v>
+        <v>Parag Relative 20 dressed &amp; other cloths</v>
       </c>
       <c r="B30" t="str">
-        <v>Miscellaneous</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C30" s="1">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="D30" s="1">
         <f>SUMIF('Payments'!$C:$C,$A30,'Payments'!$E:$E)</f>
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="E30" s="1">
         <f>C30-D30</f>
@@ -2782,55 +2802,55 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Pratap films and Photography</v>
+        <v>Petrol Glanza</v>
       </c>
       <c r="B31" t="str">
-        <v>Photography &amp; Video</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C31" s="1">
-        <v>100000</v>
+        <v>4000</v>
       </c>
       <c r="D31" s="1">
         <f>SUMIF('Payments'!$C:$C,$A31,'Payments'!$E:$E)</f>
-        <v>20000</v>
+        <v>4000</v>
       </c>
       <c r="E31" s="1">
         <f>C31-D31</f>
-        <v>80000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Pravin Masale</v>
+        <v>Pratap films and Photography</v>
       </c>
       <c r="B32" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Photography &amp; Video</v>
       </c>
       <c r="C32" s="1">
-        <v>3345</v>
+        <v>100000</v>
       </c>
       <c r="D32" s="1">
         <f>SUMIF('Payments'!$C:$C,$A32,'Payments'!$E:$E)</f>
-        <v>3345</v>
+        <v>20000</v>
       </c>
       <c r="E32" s="1">
         <f>C32-D32</f>
-        <v>0</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Prewedding shoot expences(lunch, fuel and other)</v>
+        <v>Pravin Masale</v>
       </c>
       <c r="B33" t="str">
-        <v>Miscellaneous</v>
+        <v>Food &amp; Catering</v>
       </c>
       <c r="C33" s="1">
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="D33" s="1">
         <f>SUMIF('Payments'!$C:$C,$A33,'Payments'!$E:$E)</f>
-        <v>11840</v>
+        <v>3345</v>
       </c>
       <c r="E33" s="1">
         <f>C33-D33</f>
@@ -2839,17 +2859,17 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Shireen Dress</v>
+        <v>Prewedding shoot expences(lunch, fuel and other)</v>
       </c>
       <c r="B34" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Miscellaneous</v>
       </c>
       <c r="C34" s="1">
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="D34" s="1">
         <f>SUMIF('Payments'!$C:$C,$A34,'Payments'!$E:$E)</f>
-        <v>2000</v>
+        <v>11840</v>
       </c>
       <c r="E34" s="1">
         <f>C34-D34</f>
@@ -2858,55 +2878,55 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Soyarik mangal karyalay</v>
+        <v>Shireen Dress</v>
       </c>
       <c r="B35" t="str">
-        <v>Venue &amp; Hall</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C35" s="1">
-        <v>105000</v>
+        <v>2000</v>
       </c>
       <c r="D35" s="1">
         <f>SUMIF('Payments'!$C:$C,$A35,'Payments'!$E:$E)</f>
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="E35" s="1">
         <f>C35-D35</f>
-        <v>90000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Star Bazaar - Prewedding dress</v>
+        <v>Soyarik mangal karyalay</v>
       </c>
       <c r="B36" t="str">
-        <v>Clothing &amp; Jewellery</v>
+        <v>Venue &amp; Hall</v>
       </c>
       <c r="C36" s="1">
-        <v>6190</v>
+        <v>105000</v>
       </c>
       <c r="D36" s="1">
         <f>SUMIF('Payments'!$C:$C,$A36,'Payments'!$E:$E)</f>
-        <v>6190</v>
+        <v>15000</v>
       </c>
       <c r="E36" s="1">
         <f>C36-D36</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Tushar Traders Oil</v>
+        <v>Star Bazaar - Prewedding dress</v>
       </c>
       <c r="B37" t="str">
-        <v>Food &amp; Catering</v>
+        <v>Clothing &amp; Jewellery</v>
       </c>
       <c r="C37" s="1">
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="D37" s="1">
         <f>SUMIF('Payments'!$C:$C,$A37,'Payments'!$E:$E)</f>
-        <v>5100</v>
+        <v>6190</v>
       </c>
       <c r="E37" s="1">
         <f>C37-D37</f>
@@ -2915,24 +2935,43 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
+        <v>Tushar Traders Oil</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Food &amp; Catering</v>
+      </c>
+      <c r="C38" s="1">
+        <v>5100</v>
+      </c>
+      <c r="D38" s="1">
+        <f>SUMIF('Payments'!$C:$C,$A38,'Payments'!$E:$E)</f>
+        <v>5100</v>
+      </c>
+      <c r="E38" s="1">
+        <f>C38-D38</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
         <v>Total</v>
       </c>
-      <c r="C38" s="1">
-        <f>SUM(C2:C37)</f>
-        <v>1127466</v>
-      </c>
-      <c r="D38" s="1">
-        <f>SUM(D2:D37)</f>
+      <c r="C39" s="1">
+        <f>SUM(C2:C38)</f>
+        <v>1128266</v>
+      </c>
+      <c r="D39" s="1">
+        <f>SUM(D2:D38)</f>
         <v>296466</v>
       </c>
-      <c r="E38" s="1">
-        <f>SUM(E2:E37)</f>
-        <v>831000</v>
+      <c r="E39" s="1">
+        <f>SUM(E2:E38)</f>
+        <v>831800</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record payment: ₹800.00 by Asif Sayyed (Son) for Colour & plumber
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -9,7 +9,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Budget'!A1:F38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Payments'!A1:H40</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1187,7 +1187,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2163,19 +2163,19 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>0bd24ffb</v>
+        <v>e53fce6e</v>
       </c>
       <c r="B38" t="str">
-        <v>aaedf833</v>
+        <v>2a74d868</v>
       </c>
       <c r="C38" t="str">
-        <v>Aluminum Shop Partition</v>
+        <v>Colour &amp; plumber</v>
       </c>
       <c r="D38" s="3">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="E38" s="1">
-        <v>15000</v>
+        <v>800</v>
       </c>
       <c r="F38" t="str">
         <v>Asif Sayyed (Son)</v>
@@ -2184,39 +2184,65 @@
         <v>UPI</v>
       </c>
       <c r="H38" t="str">
-        <v>Paid Advance</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
+        <v>0bd24ffb</v>
+      </c>
+      <c r="B39" t="str">
+        <v>aaedf833</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Aluminum Shop Partition</v>
+      </c>
+      <c r="D39" s="3">
+        <v>46271</v>
+      </c>
+      <c r="E39" s="1">
+        <v>15000</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Asif Sayyed (Son)</v>
+      </c>
+      <c r="G39" t="str">
+        <v>UPI</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Paid Advance</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
         <v>a1d6ea2f</v>
       </c>
-      <c r="B39" t="str">
+      <c r="B40" t="str">
         <v>30b69ec5</v>
       </c>
-      <c r="C39" t="str">
+      <c r="C40" t="str">
         <v>Mummy sadi</v>
       </c>
-      <c r="D39" s="3">
+      <c r="D40" s="3">
         <v>46272</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E40" s="1">
         <v>1600</v>
       </c>
-      <c r="F39" t="str">
+      <c r="F40" t="str">
         <v>Umar Sayyed (Father)</v>
       </c>
-      <c r="G39" t="str">
+      <c r="G40" t="str">
         <v>Cash</v>
       </c>
-      <c r="H39" t="str">
+      <c r="H40" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H39"/>
+  <autoFilter ref="A1:H40"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H40"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2451,11 +2477,11 @@
       </c>
       <c r="D12" s="1">
         <f>SUMIF('Payments'!$C:$C,$A12,'Payments'!$E:$E)</f>
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="E12" s="1">
         <f>C12-D12</f>
-        <v>800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2962,11 +2988,11 @@
       </c>
       <c r="D39" s="1">
         <f>SUM(D2:D38)</f>
-        <v>296466</v>
+        <v>297266</v>
       </c>
       <c r="E39" s="1">
         <f>SUM(E2:E38)</f>
-        <v>831800</v>
+        <v>831000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>